<commit_message>
added weigh1_numbers 2 to meta data
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="117">
   <si>
     <t>nspp</t>
   </si>
@@ -364,13 +364,19 @@
   </si>
   <si>
     <t>NOTE: Most objects are ordered by species code if not specified</t>
+  </si>
+  <si>
+    <t>weight1_Numbers2</t>
+  </si>
+  <si>
+    <t>Is the observation in weight (kg) set as 1, if the observation is in numbers caught, set as 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -501,6 +507,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -847,9 +860,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1456,6 +1470,12 @@
       <c r="D14" t="s">
         <v>12</v>
       </c>
+      <c r="F14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G14" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">

</xml_diff>

<commit_message>
Added ability to estimate srv sigma and changed minage
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="133">
   <si>
     <t>nspp</t>
   </si>
@@ -150,9 +150,6 @@
     <t>Start year of the hindcast</t>
   </si>
   <si>
-    <t>Number of ages of each species included in the hindcast</t>
-  </si>
-  <si>
     <t>Number of lengths of each species included in the hindcast</t>
   </si>
   <si>
@@ -321,9 +318,6 @@
     <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic</t>
   </si>
   <si>
-    <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2. Not used otherwise</t>
-  </si>
-  <si>
     <t>Units used for survey: 1 = kg; 2 = numbers</t>
   </si>
   <si>
@@ -370,13 +364,67 @@
   </si>
   <si>
     <t>Minimum age of each species included in the hindcast</t>
+  </si>
+  <si>
+    <t>weight1_Numbers2</t>
+  </si>
+  <si>
+    <t>Is the observation in weight (kg) set as 1, if the observation is in numbers caught, set as 2</t>
+  </si>
+  <si>
+    <t>Number of ages of each species included in the hindcast. Includes age 0 if minage = 0</t>
+  </si>
+  <si>
+    <t>Number of ages (starting from minage) to estimate non-parametric selectivity for Selectivity = 2. Not used otherwise</t>
+  </si>
+  <si>
+    <t>Estimate_sigma_catch</t>
+  </si>
+  <si>
+    <t>Estimate_sigma_index</t>
+  </si>
+  <si>
+    <t>Should CEATTLE estimate the variance associated with the catch time series (yes = 1; no = 0). If 0, uses the CV from fsh_biom.</t>
+  </si>
+  <si>
+    <t>Should CEATTLE estimate the variance associated with the survey index time series (yes = 1; no = 0). If 0, uses the CV from srv_biom.</t>
+  </si>
+  <si>
+    <t>Sigma_catch_prior</t>
+  </si>
+  <si>
+    <t>Prior for sigma_catch to be used if Estimate_sigma_catch = 1</t>
+  </si>
+  <si>
+    <t>Sigma_index_prior</t>
+  </si>
+  <si>
+    <t>Prior for sigma_catch to be used if Estimate_sigma_index = 1</t>
+  </si>
+  <si>
+    <t>sigma_rec_prior</t>
+  </si>
+  <si>
+    <t>Prior to be used for estimating the standard deviation around recruitment deviates. Is the starting value if random_rec = TRUE when using fit_mod.</t>
+  </si>
+  <si>
+    <t>projyr</t>
+  </si>
+  <si>
+    <t>End year of the forecast</t>
+  </si>
+  <si>
+    <t>proj_F</t>
+  </si>
+  <si>
+    <t>Projected F rate for forecast of each fishery</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -507,6 +555,19 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -853,9 +914,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1177,13 +1242,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="119.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="2"/>
+    <col min="6" max="6" width="23.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1191,713 +1259,777 @@
         <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G3" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="C4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
         <v>42</v>
       </c>
-      <c r="D3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B43" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
         <v>45</v>
       </c>
-      <c r="D4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" t="s">
-        <v>111</v>
-      </c>
-      <c r="G5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>115</v>
-      </c>
-      <c r="C6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B46" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
         <v>46</v>
       </c>
-      <c r="D8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>91</v>
-      </c>
-      <c r="G9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" t="s">
-        <v>93</v>
-      </c>
-      <c r="G11" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>94</v>
-      </c>
-      <c r="G12" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>95</v>
-      </c>
-      <c r="G13" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" t="s">
-        <v>63</v>
-      </c>
-      <c r="D24" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" t="s">
-        <v>64</v>
-      </c>
-      <c r="D25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>23</v>
-      </c>
-      <c r="C26" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" t="s">
-        <v>75</v>
-      </c>
-      <c r="D28" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" t="s">
-        <v>27</v>
-      </c>
-      <c r="C30" t="s">
-        <v>107</v>
-      </c>
-      <c r="D30" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" t="s">
-        <v>28</v>
-      </c>
-      <c r="C31" t="s">
-        <v>70</v>
-      </c>
-      <c r="D31" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" t="s">
-        <v>29</v>
-      </c>
-      <c r="C32" t="s">
-        <v>71</v>
-      </c>
-      <c r="D32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" t="s">
-        <v>30</v>
-      </c>
-      <c r="C33" t="s">
-        <v>72</v>
-      </c>
-      <c r="D33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34" t="s">
-        <v>31</v>
-      </c>
-      <c r="C34" t="s">
-        <v>72</v>
-      </c>
-      <c r="D34" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" t="s">
-        <v>72</v>
-      </c>
-      <c r="D35" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>33</v>
-      </c>
-      <c r="C36" t="s">
-        <v>72</v>
-      </c>
-      <c r="D36" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" t="s">
-        <v>34</v>
-      </c>
-      <c r="C37" t="s">
-        <v>72</v>
-      </c>
-      <c r="D37" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>35</v>
-      </c>
-      <c r="C38" t="s">
-        <v>72</v>
-      </c>
-      <c r="D38" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>36</v>
-      </c>
-      <c r="C39" t="s">
-        <v>73</v>
-      </c>
-      <c r="D39" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40" t="s">
-        <v>74</v>
-      </c>
-      <c r="D40" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
-        <v>38</v>
-      </c>
-      <c r="C41" t="s">
-        <v>76</v>
-      </c>
-      <c r="D41" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>78</v>
-      </c>
-      <c r="C42" t="s">
-        <v>82</v>
-      </c>
-      <c r="D42" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="s">
-        <v>79</v>
-      </c>
-      <c r="C43" t="s">
-        <v>83</v>
-      </c>
-      <c r="D43" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="s">
+      <c r="B47" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C47" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D47" s="2" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>81</v>
-      </c>
-      <c r="C45" t="s">
-        <v>85</v>
-      </c>
-      <c r="D45" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added analytical q for surveys and analytical sigma
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="127">
   <si>
     <t>nspp</t>
   </si>
@@ -336,9 +336,6 @@
     <t>Age transition matrix (e.g. Age Length Key or ALK) index to use for derived quantitied</t>
   </si>
   <si>
-    <t>Estimate catchability? (0 = no; 1 = yes)</t>
-  </si>
-  <si>
     <t>Starting value or fixed value for catchability</t>
   </si>
   <si>
@@ -370,6 +367,39 @@
   </si>
   <si>
     <t>Is the observation in weight (kg) set as 1, if the observation is in numbers caught, set as 2</t>
+  </si>
+  <si>
+    <t>Estimate catchability? (0 = no; 1 = yes, 2 = analytical from Ludwig and Walters 1994)</t>
+  </si>
+  <si>
+    <t>Estimate_sigma_index</t>
+  </si>
+  <si>
+    <t>Estimate survey variance (0 = use CV from srv_biom, 1 = yes, 2 = analytically estimate following (Ludwig and Walters 1994)</t>
+  </si>
+  <si>
+    <t>Sigma_index_prior</t>
+  </si>
+  <si>
+    <t>Starting value to be used if Estimate_sigma_index = 1</t>
+  </si>
+  <si>
+    <t>Estimate_sigma_catch</t>
+  </si>
+  <si>
+    <t>Estimate fishery variance (0 = use CV from srv_biom, 1 = yes, 2 = analytically estimate following (Ludwig and Walters 1994)</t>
+  </si>
+  <si>
+    <t>Sigma_catch_prior</t>
+  </si>
+  <si>
+    <t>Starting value to be used if Estimate_sigma_catch = 1</t>
+  </si>
+  <si>
+    <t>NOTE: Lengths are index 1 through nlenths</t>
+  </si>
+  <si>
+    <t>NOTE: Columns for ages are index by 1 trhough nages</t>
   </si>
 </sst>
 </file>
@@ -860,10 +890,18 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1208,10 +1246,10 @@
         <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>40</v>
@@ -1271,10 +1309,10 @@
         <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1291,10 +1329,10 @@
         <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1434,7 +1472,7 @@
         <v>94</v>
       </c>
       <c r="G12" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1450,11 +1488,11 @@
       <c r="D13" t="s">
         <v>11</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>95</v>
       </c>
       <c r="G13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1470,11 +1508,11 @@
       <c r="D14" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G14" t="s">
         <v>115</v>
-      </c>
-      <c r="G14" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1490,6 +1528,12 @@
       <c r="D15" t="s">
         <v>13</v>
       </c>
+      <c r="F15" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1504,11 +1548,14 @@
       <c r="D16" t="s">
         <v>14</v>
       </c>
-      <c r="F16" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1521,8 +1568,14 @@
       <c r="D17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F17" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1535,8 +1588,14 @@
       <c r="D18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1550,7 +1609,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1564,7 +1623,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1578,7 +1637,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1592,7 +1651,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1606,7 +1665,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1620,7 +1679,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1633,8 +1692,11 @@
       <c r="D25" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1647,8 +1709,11 @@
       <c r="D26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1661,8 +1726,11 @@
       <c r="D27" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1676,7 +1744,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1684,13 +1752,13 @@
         <v>27</v>
       </c>
       <c r="C29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D29" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1704,7 +1772,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1718,7 +1786,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
added tv q and sel to build params and map and data
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10309"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grant Adams\Documents\GitHub\Rceattle\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F15347-0179-E14B-9092-1C6EA2FC6A68}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="139">
   <si>
     <t>nspp</t>
   </si>
@@ -400,13 +401,49 @@
   </si>
   <si>
     <t>NOTE: Columns for ages are index by 1 trhough nages</t>
+  </si>
+  <si>
+    <t>Time_varying_sel</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect.</t>
+  </si>
+  <si>
+    <t>Sel_sd_prior</t>
+  </si>
+  <si>
+    <t>The sd to use for the random walk of time varying selectivity if set to 1</t>
+  </si>
+  <si>
+    <t>Time_varying_q</t>
+  </si>
+  <si>
+    <t>Q_sd_prior</t>
+  </si>
+  <si>
+    <t>The sd to use for the random walk of time varying q if set to 1</t>
+  </si>
+  <si>
+    <t>Wether a time-varying q should be estimated. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect.</t>
+  </si>
+  <si>
+    <t>Selectivity_index</t>
+  </si>
+  <si>
+    <t>index to use if selectivitys of different surveys are to be the same</t>
+  </si>
+  <si>
+    <t>Q_index</t>
+  </si>
+  <si>
+    <t>index to use if catchability coefficients are to be set the same</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1222,17 +1259,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="119.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.5" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -1255,7 +1292,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1275,7 +1312,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1295,7 +1332,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1315,7 +1352,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1335,7 +1372,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1355,7 +1392,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1375,7 +1412,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1395,7 +1432,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1415,7 +1452,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1435,7 +1472,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1455,7 +1492,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1475,7 +1512,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1495,7 +1532,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1515,7 +1552,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1535,7 +1572,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1555,7 +1592,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1575,7 +1612,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1595,7 +1632,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1608,8 +1645,14 @@
       <c r="D19" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>127</v>
+      </c>
+      <c r="G19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1622,8 +1665,14 @@
       <c r="D20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G20" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1636,8 +1685,14 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
+        <v>131</v>
+      </c>
+      <c r="G21" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1650,8 +1705,14 @@
       <c r="D22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>132</v>
+      </c>
+      <c r="G22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1664,8 +1725,14 @@
       <c r="D23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>135</v>
+      </c>
+      <c r="G23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1678,8 +1745,14 @@
       <c r="D24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>137</v>
+      </c>
+      <c r="G24" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1696,7 +1769,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1713,7 +1786,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1730,7 +1803,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1744,7 +1817,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1758,7 +1831,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1772,7 +1845,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1786,7 +1859,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1800,7 +1873,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1814,7 +1887,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1828,7 +1901,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1842,7 +1915,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1856,7 +1929,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1870,7 +1943,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1884,7 +1957,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1898,7 +1971,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1912,7 +1985,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1926,7 +1999,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1940,7 +2013,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1954,7 +2027,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4">
       <c r="A44">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
updated names of sigma index
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F15347-0179-E14B-9092-1C6EA2FC6A68}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3E6C21-7787-2F40-8A10-10FEFA542231}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -373,15 +373,9 @@
     <t>Estimate catchability? (0 = no; 1 = yes, 2 = analytical from Ludwig and Walters 1994)</t>
   </si>
   <si>
-    <t>Estimate_sigma_index</t>
-  </si>
-  <si>
     <t>Estimate survey variance (0 = use CV from srv_biom, 1 = yes, 2 = analytically estimate following (Ludwig and Walters 1994)</t>
   </si>
   <si>
-    <t>Sigma_index_prior</t>
-  </si>
-  <si>
     <t>Starting value to be used if Estimate_sigma_index = 1</t>
   </si>
   <si>
@@ -400,9 +394,6 @@
     <t>NOTE: Lengths are index 1 through nlenths</t>
   </si>
   <si>
-    <t>NOTE: Columns for ages are index by 1 trhough nages</t>
-  </si>
-  <si>
     <t>Time_varying_sel</t>
   </si>
   <si>
@@ -437,6 +428,15 @@
   </si>
   <si>
     <t>index to use if catchability coefficients are to be set the same</t>
+  </si>
+  <si>
+    <t>Sigma_survey_prior</t>
+  </si>
+  <si>
+    <t>Estimate_sigma_survey</t>
+  </si>
+  <si>
+    <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
   </si>
 </sst>
 </file>
@@ -1566,10 +1566,10 @@
         <v>13</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G15" t="s">
         <v>117</v>
-      </c>
-      <c r="G15" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1586,10 +1586,10 @@
         <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="G16" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1606,10 +1606,10 @@
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G17" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1626,10 +1626,10 @@
         <v>16</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G18" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1646,10 +1646,10 @@
         <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G19" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1666,10 +1666,10 @@
         <v>18</v>
       </c>
       <c r="F20" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G20" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1686,10 +1686,10 @@
         <v>19</v>
       </c>
       <c r="F21" t="s">
+        <v>128</v>
+      </c>
+      <c r="G21" t="s">
         <v>131</v>
-      </c>
-      <c r="G21" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1706,10 +1706,10 @@
         <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G22" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1726,10 +1726,10 @@
         <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="G23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1746,10 +1746,10 @@
         <v>22</v>
       </c>
       <c r="F24" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G24" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1765,9 +1765,6 @@
       <c r="D25" t="s">
         <v>23</v>
       </c>
-      <c r="F25" t="s">
-        <v>113</v>
-      </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26">
@@ -1782,9 +1779,6 @@
       <c r="D26" t="s">
         <v>24</v>
       </c>
-      <c r="F26" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27">
@@ -1799,9 +1793,6 @@
       <c r="D27" t="s">
         <v>68</v>
       </c>
-      <c r="F27" t="s">
-        <v>126</v>
-      </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28">
@@ -1830,6 +1821,9 @@
       <c r="D29" t="s">
         <v>68</v>
       </c>
+      <c r="F29" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30">
@@ -1844,6 +1838,9 @@
       <c r="D30" t="s">
         <v>68</v>
       </c>
+      <c r="F30" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31">
@@ -1857,6 +1854,9 @@
       </c>
       <c r="D31" t="s">
         <v>68</v>
+      </c>
+      <c r="F31" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="32" spans="1:7">

</xml_diff>

<commit_message>
updated parameters and time varying selectivity and catachbility in cpp, need to change map function to deal with blocks and such
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10309"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grant Adams\Documents\GitHub\Rceattle\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3E6C21-7787-2F40-8A10-10FEFA542231}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="465" windowWidth="25605" windowHeight="12345"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="139">
   <si>
     <t>nspp</t>
   </si>
@@ -397,9 +396,6 @@
     <t>Time_varying_sel</t>
   </si>
   <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect.</t>
-  </si>
-  <si>
     <t>Sel_sd_prior</t>
   </si>
   <si>
@@ -415,9 +411,6 @@
     <t>The sd to use for the random walk of time varying q if set to 1</t>
   </si>
   <si>
-    <t>Wether a time-varying q should be estimated. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect.</t>
-  </si>
-  <si>
     <t>Selectivity_index</t>
   </si>
   <si>
@@ -437,13 +430,19 @@
   </si>
   <si>
     <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
+  </si>
+  <si>
+    <t>Wether a time-varying q should be estimated. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penalty</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1259,17 +1258,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="119.5" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -1292,7 +1291,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1312,7 +1311,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1332,7 +1331,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1352,7 +1351,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1372,7 +1371,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1392,7 +1391,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1412,7 +1411,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1432,7 +1431,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1452,7 +1451,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1472,7 +1471,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1492,7 +1491,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1512,7 +1511,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1532,7 +1531,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1552,7 +1551,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1566,13 +1565,13 @@
         <v>13</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G15" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1586,13 +1585,13 @@
         <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1612,7 +1611,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1632,7 +1631,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1649,10 +1648,10 @@
         <v>124</v>
       </c>
       <c r="G19" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1666,13 +1665,13 @@
         <v>18</v>
       </c>
       <c r="F20" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" t="s">
         <v>126</v>
       </c>
-      <c r="G20" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1686,13 +1685,13 @@
         <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G21" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1706,13 +1705,13 @@
         <v>20</v>
       </c>
       <c r="F22" t="s">
+        <v>128</v>
+      </c>
+      <c r="G22" t="s">
         <v>129</v>
       </c>
-      <c r="G22" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1726,13 +1725,13 @@
         <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G23" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1746,13 +1745,13 @@
         <v>22</v>
       </c>
       <c r="F24" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G24" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1766,7 +1765,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1780,7 +1779,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1794,7 +1793,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1808,7 +1807,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1825,7 +1824,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1842,7 +1841,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1856,10 +1855,10 @@
         <v>68</v>
       </c>
       <c r="F31" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1873,7 +1872,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1887,7 +1886,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1901,7 +1900,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1915,7 +1914,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1929,7 +1928,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1943,7 +1942,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1957,7 +1956,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1971,7 +1970,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1985,7 +1984,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1999,7 +1998,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2013,7 +2012,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2027,7 +2026,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Added polygon plots for survey and age comps
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="0" yWindow="465" windowWidth="25605" windowHeight="12345"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="139">
   <si>
     <t>nspp</t>
   </si>
@@ -372,15 +372,9 @@
     <t>Estimate catchability? (0 = no; 1 = yes, 2 = analytical from Ludwig and Walters 1994)</t>
   </si>
   <si>
-    <t>Estimate_sigma_index</t>
-  </si>
-  <si>
     <t>Estimate survey variance (0 = use CV from srv_biom, 1 = yes, 2 = analytically estimate following (Ludwig and Walters 1994)</t>
   </si>
   <si>
-    <t>Sigma_index_prior</t>
-  </si>
-  <si>
     <t>Starting value to be used if Estimate_sigma_index = 1</t>
   </si>
   <si>
@@ -399,7 +393,49 @@
     <t>NOTE: Lengths are index 1 through nlenths</t>
   </si>
   <si>
-    <t>NOTE: Columns for ages are index by 1 trhough nages</t>
+    <t>Time_varying_sel</t>
+  </si>
+  <si>
+    <t>Sel_sd_prior</t>
+  </si>
+  <si>
+    <t>The sd to use for the random walk of time varying selectivity if set to 1</t>
+  </si>
+  <si>
+    <t>Time_varying_q</t>
+  </si>
+  <si>
+    <t>Q_sd_prior</t>
+  </si>
+  <si>
+    <t>The sd to use for the random walk of time varying q if set to 1</t>
+  </si>
+  <si>
+    <t>Selectivity_index</t>
+  </si>
+  <si>
+    <t>index to use if selectivitys of different surveys are to be the same</t>
+  </si>
+  <si>
+    <t>Q_index</t>
+  </si>
+  <si>
+    <t>index to use if catchability coefficients are to be set the same</t>
+  </si>
+  <si>
+    <t>Sigma_survey_prior</t>
+  </si>
+  <si>
+    <t>Estimate_sigma_survey</t>
+  </si>
+  <si>
+    <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
+  </si>
+  <si>
+    <t>Wether a time-varying q should be estimated. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penalty</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality</t>
   </si>
 </sst>
 </file>
@@ -1224,10 +1260,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="119.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.42578125" customWidth="1"/>
     <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -1529,10 +1565,10 @@
         <v>13</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G15" t="s">
         <v>117</v>
-      </c>
-      <c r="G15" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1549,10 +1585,10 @@
         <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="G16" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1569,10 +1605,10 @@
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G17" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1589,10 +1625,10 @@
         <v>16</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G18" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1608,6 +1644,12 @@
       <c r="D19" t="s">
         <v>17</v>
       </c>
+      <c r="F19" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
@@ -1622,6 +1664,12 @@
       <c r="D20" t="s">
         <v>18</v>
       </c>
+      <c r="F20" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
@@ -1636,6 +1684,12 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
+      <c r="F21" t="s">
+        <v>127</v>
+      </c>
+      <c r="G21" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
@@ -1650,6 +1704,12 @@
       <c r="D22" t="s">
         <v>20</v>
       </c>
+      <c r="F22" t="s">
+        <v>128</v>
+      </c>
+      <c r="G22" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
@@ -1664,6 +1724,12 @@
       <c r="D23" t="s">
         <v>21</v>
       </c>
+      <c r="F23" t="s">
+        <v>130</v>
+      </c>
+      <c r="G23" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
@@ -1678,6 +1744,12 @@
       <c r="D24" t="s">
         <v>22</v>
       </c>
+      <c r="F24" t="s">
+        <v>132</v>
+      </c>
+      <c r="G24" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
@@ -1692,9 +1764,6 @@
       <c r="D25" t="s">
         <v>23</v>
       </c>
-      <c r="F25" t="s">
-        <v>113</v>
-      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
@@ -1709,9 +1778,6 @@
       <c r="D26" t="s">
         <v>24</v>
       </c>
-      <c r="F26" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
@@ -1726,9 +1792,6 @@
       <c r="D27" t="s">
         <v>68</v>
       </c>
-      <c r="F27" t="s">
-        <v>126</v>
-      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
@@ -1757,6 +1820,9 @@
       <c r="D29" t="s">
         <v>68</v>
       </c>
+      <c r="F29" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
@@ -1771,6 +1837,9 @@
       <c r="D30" t="s">
         <v>68</v>
       </c>
+      <c r="F30" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
@@ -1784,6 +1853,9 @@
       </c>
       <c r="D31" t="s">
         <v>68</v>
+      </c>
+      <c r="F31" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Cleans data and updated naming
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="139">
   <si>
     <t>nspp</t>
   </si>
@@ -294,9 +294,6 @@
     <t>Nselages</t>
   </si>
   <si>
-    <t>Catch_units</t>
-  </si>
-  <si>
     <t>Weight_index</t>
   </si>
   <si>
@@ -324,9 +321,6 @@
     <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2. Not used otherwise</t>
   </si>
   <si>
-    <t>Units used for survey: 1 = kg; 2 = numbers</t>
-  </si>
-  <si>
     <t>Weight-at-age (wt) index to use for calculation of derived quantities</t>
   </si>
   <si>
@@ -436,6 +430,12 @@
   </si>
   <si>
     <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality</t>
+  </si>
+  <si>
+    <t>Fit_0no_1yes</t>
+  </si>
+  <si>
+    <t>Index of wether data should be included in the likelihood and associated parameters estimated.</t>
   </si>
 </sst>
 </file>
@@ -1282,10 +1282,10 @@
         <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>40</v>
@@ -1308,7 +1308,7 @@
         <v>86</v>
       </c>
       <c r="G2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1328,7 +1328,7 @@
         <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1345,10 +1345,10 @@
         <v>60</v>
       </c>
       <c r="F4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" t="s">
         <v>109</v>
-      </c>
-      <c r="G4" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1365,10 +1365,10 @@
         <v>60</v>
       </c>
       <c r="F5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" t="s">
         <v>110</v>
-      </c>
-      <c r="G5" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1388,7 +1388,7 @@
         <v>88</v>
       </c>
       <c r="G6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1405,10 +1405,10 @@
         <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="G7" t="s">
-        <v>99</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1419,16 +1419,16 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D8" t="s">
         <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1445,10 +1445,10 @@
         <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1464,11 +1464,11 @@
       <c r="D10" t="s">
         <v>60</v>
       </c>
-      <c r="F10" t="s">
-        <v>92</v>
+      <c r="F10" s="3" t="s">
+        <v>112</v>
       </c>
       <c r="G10" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1485,10 +1485,10 @@
         <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1505,10 +1505,10 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G12" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1524,11 +1524,11 @@
       <c r="D13" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>95</v>
+      <c r="F13" t="s">
+        <v>93</v>
       </c>
       <c r="G13" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1544,11 +1544,11 @@
       <c r="D14" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>114</v>
+      <c r="F14" s="2" t="s">
+        <v>94</v>
       </c>
       <c r="G14" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1565,10 +1565,10 @@
         <v>13</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1585,10 +1585,10 @@
         <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G16" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1605,10 +1605,10 @@
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G17" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1625,10 +1625,10 @@
         <v>16</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G18" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1645,10 +1645,10 @@
         <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G19" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1665,10 +1665,10 @@
         <v>18</v>
       </c>
       <c r="F20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G20" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1685,10 +1685,10 @@
         <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1705,10 +1705,10 @@
         <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G22" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1725,10 +1725,10 @@
         <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G23" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1745,10 +1745,10 @@
         <v>22</v>
       </c>
       <c r="F24" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1815,13 +1815,13 @@
         <v>27</v>
       </c>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
         <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1838,7 +1838,7 @@
         <v>68</v>
       </c>
       <c r="F30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1855,7 +1855,7 @@
         <v>68</v>
       </c>
       <c r="F31" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added ssb bits following dorn
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="153">
   <si>
     <t>nspp</t>
   </si>
@@ -436,6 +436,48 @@
   </si>
   <si>
     <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality</t>
+  </si>
+  <si>
+    <t>projyr</t>
+  </si>
+  <si>
+    <t>End year of the forecast</t>
+  </si>
+  <si>
+    <t>nsex</t>
+  </si>
+  <si>
+    <t>spawn_month</t>
+  </si>
+  <si>
+    <t>Spawning month of the population to adjust the numbers spawning</t>
+  </si>
+  <si>
+    <t>R_sexr</t>
+  </si>
+  <si>
+    <t>Percent of recruitment that is female (ignored if nsex = 1)</t>
+  </si>
+  <si>
+    <t>Number of sexes to model in the population (1 = combined/1sex, 2 = models both female/male)</t>
+  </si>
+  <si>
+    <t>minage</t>
+  </si>
+  <si>
+    <t>Minimum age for each population (i.e.does recruitment correspond to age 0, 1, 2?)</t>
+  </si>
+  <si>
+    <t>ssb_wt_index</t>
+  </si>
+  <si>
+    <t>Weight-at-age (wt) index to use for calculation of each species spawning biomass</t>
+  </si>
+  <si>
+    <t>sigma_rec_prior</t>
+  </si>
+  <si>
+    <t>Standard deviation to use for recruitment</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1301,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -1356,10 +1398,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>140</v>
       </c>
       <c r="D5" t="s">
         <v>60</v>
@@ -1376,10 +1418,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
         <v>60</v>
@@ -1396,10 +1438,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>143</v>
       </c>
       <c r="D7" t="s">
         <v>60</v>
@@ -1416,10 +1458,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>144</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="D8" t="s">
         <v>60</v>
@@ -1436,10 +1478,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
         <v>60</v>
@@ -1456,10 +1498,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>147</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>148</v>
       </c>
       <c r="D10" t="s">
         <v>60</v>
@@ -1476,13 +1518,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
         <v>93</v>
@@ -1496,13 +1538,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="F12" t="s">
         <v>94</v>
@@ -1516,13 +1558,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>95</v>
@@ -1536,13 +1578,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>103</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>114</v>
@@ -1556,13 +1598,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>151</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>152</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>135</v>
@@ -1576,13 +1618,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>134</v>
@@ -1596,13 +1638,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>119</v>
@@ -1613,16 +1655,16 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>121</v>
@@ -1633,16 +1675,16 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F19" t="s">
         <v>124</v>
@@ -1653,16 +1695,16 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F20" t="s">
         <v>125</v>
@@ -1673,16 +1715,16 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F21" t="s">
         <v>127</v>
@@ -1693,16 +1735,16 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F22" t="s">
         <v>128</v>
@@ -1713,16 +1755,16 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
         <v>130</v>
@@ -1733,16 +1775,16 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F24" t="s">
         <v>132</v>
@@ -1753,72 +1795,72 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="D26" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C27" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="D29" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="F29" t="s">
         <v>113</v>
@@ -1826,16 +1868,16 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D30" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="F30" t="s">
         <v>123</v>
@@ -1843,16 +1885,16 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="F31" t="s">
         <v>136</v>
@@ -1860,41 +1902,41 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C32" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D33" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C34" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D34" t="s">
         <v>68</v>
@@ -1902,13 +1944,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
         <v>68</v>
@@ -1916,13 +1958,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="D36" t="s">
         <v>68</v>
@@ -1930,13 +1972,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
         <v>68</v>
@@ -1944,99 +1986,197 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="C41" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="C42" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="C43" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="D43" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
+        <v>36</v>
+      </c>
+      <c r="B44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C44" t="s">
+        <v>72</v>
+      </c>
+      <c r="D44" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>37</v>
+      </c>
+      <c r="B45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" t="s">
+        <v>73</v>
+      </c>
+      <c r="D45" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>38</v>
+      </c>
+      <c r="B46" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46" t="s">
+        <v>74</v>
+      </c>
+      <c r="D46" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>39</v>
+      </c>
+      <c r="B47" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47" t="s">
+        <v>76</v>
+      </c>
+      <c r="D47" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>40</v>
+      </c>
+      <c r="B48" t="s">
+        <v>78</v>
+      </c>
+      <c r="C48" t="s">
+        <v>82</v>
+      </c>
+      <c r="D48" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>41</v>
+      </c>
+      <c r="B49" t="s">
+        <v>79</v>
+      </c>
+      <c r="C49" t="s">
+        <v>83</v>
+      </c>
+      <c r="D49" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>42</v>
+      </c>
+      <c r="B50" t="s">
+        <v>80</v>
+      </c>
+      <c r="C50" t="s">
+        <v>84</v>
+      </c>
+      <c r="D50" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
         <v>43</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B51" t="s">
         <v>81</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C51" t="s">
         <v>85</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D51" t="s">
         <v>81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
started update on sex specific model
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="155">
   <si>
     <t>nspp</t>
   </si>
@@ -478,6 +478,12 @@
   </si>
   <si>
     <t>Standard deviation to use for recruitment</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>sex codes: 0=combined; 1=use female only; 2=use male only</t>
   </si>
 </sst>
 </file>
@@ -1447,10 +1453,10 @@
         <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>89</v>
+        <v>153</v>
       </c>
       <c r="G7" t="s">
-        <v>99</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1467,10 +1473,10 @@
         <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1487,10 +1493,10 @@
         <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1507,10 +1513,10 @@
         <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1527,10 +1533,10 @@
         <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1547,10 +1553,10 @@
         <v>60</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G12" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1566,11 +1572,11 @@
       <c r="D13" t="s">
         <v>60</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>95</v>
+      <c r="F13" t="s">
+        <v>94</v>
       </c>
       <c r="G13" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1586,11 +1592,11 @@
       <c r="D14" t="s">
         <v>60</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>114</v>
+      <c r="F14" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="G14" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1606,11 +1612,11 @@
       <c r="D15" t="s">
         <v>60</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>135</v>
+      <c r="F15" s="3" t="s">
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1626,11 +1632,11 @@
       <c r="D16" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>134</v>
+      <c r="F16" s="4" t="s">
+        <v>135</v>
       </c>
       <c r="G16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1646,11 +1652,11 @@
       <c r="D17" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>119</v>
+      <c r="F17" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="G17" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1667,10 +1673,10 @@
         <v>9</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G18" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1686,11 +1692,11 @@
       <c r="D19" t="s">
         <v>10</v>
       </c>
-      <c r="F19" t="s">
-        <v>124</v>
+      <c r="F19" s="4" t="s">
+        <v>121</v>
       </c>
       <c r="G19" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1707,10 +1713,10 @@
         <v>11</v>
       </c>
       <c r="F20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G20" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1727,10 +1733,10 @@
         <v>12</v>
       </c>
       <c r="F21" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G21" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1747,10 +1753,10 @@
         <v>13</v>
       </c>
       <c r="F22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G22" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1767,10 +1773,10 @@
         <v>14</v>
       </c>
       <c r="F23" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G23" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1787,10 +1793,10 @@
         <v>15</v>
       </c>
       <c r="F24" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1805,6 +1811,12 @@
       </c>
       <c r="D25" t="s">
         <v>16</v>
+      </c>
+      <c r="F25" t="s">
+        <v>132</v>
+      </c>
+      <c r="G25" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated non-parametric selectivity penalties
Updated choice of non-parametric selectivity penalties. They are now set using Time_varying_sel and Sel_sd_prior. At some point I should change the naming convention to Sel_setting_1, Sel_setting_2 or similar
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10810"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grant Adams\Documents\GitHub\Rceattle\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0BF229-F42D-1249-8354-90EAE7EBF434}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="465" windowWidth="25605" windowHeight="12345"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="161">
   <si>
     <t>nspp</t>
   </si>
@@ -201,9 +202,6 @@
     <t>Weight-at-age (wt) to use for calculation of derived quantities (SSB, Consumption/Ration, Suitability, Total Catch, Survey Biomass, etc). Can have multiple weight-at-age data-sets for each species, but must be full for all years of the hindcast.</t>
   </si>
   <si>
-    <t>control</t>
-  </si>
-  <si>
     <t>Sheet location</t>
   </si>
   <si>
@@ -225,9 +223,6 @@
     <t>data_list Object name</t>
   </si>
   <si>
-    <t>bioenergetics_control</t>
-  </si>
-  <si>
     <t>This scales the maximum consumption used for ration for each species; Pvalue is in Cmax*fT*Pvalue*Page</t>
   </si>
   <si>
@@ -252,9 +247,6 @@
     <t>Annual relative foraging rate by age</t>
   </si>
   <si>
-    <t>Temp_data</t>
-  </si>
-  <si>
     <t>UobsAge</t>
   </si>
   <si>
@@ -279,12 +271,6 @@
     <t>Stomach proportion by weight for each predator, prey, predator length prey length combination. Can also be year specific by including the column, "Year"</t>
   </si>
   <si>
-    <t>Survey_name</t>
-  </si>
-  <si>
-    <t>Survey_code</t>
-  </si>
-  <si>
     <t>Species</t>
   </si>
   <si>
@@ -306,15 +292,6 @@
     <t>Estimate_q</t>
   </si>
   <si>
-    <t>log_q_start</t>
-  </si>
-  <si>
-    <t>Name of survey</t>
-  </si>
-  <si>
-    <t>Index of survey ACROSS species</t>
-  </si>
-  <si>
     <t>Species number</t>
   </si>
   <si>
@@ -348,18 +325,6 @@
     <t>Column names</t>
   </si>
   <si>
-    <t>Fishery_name</t>
-  </si>
-  <si>
-    <t>Fishery_code</t>
-  </si>
-  <si>
-    <t>Name of fishery</t>
-  </si>
-  <si>
-    <t>Index of fishery ACROSS species</t>
-  </si>
-  <si>
     <t>NOTE: Most objects are ordered by species code if not specified</t>
   </si>
   <si>
@@ -378,15 +343,9 @@
     <t>Starting value to be used if Estimate_sigma_index = 1</t>
   </si>
   <si>
-    <t>Estimate_sigma_catch</t>
-  </si>
-  <si>
     <t>Estimate fishery variance (0 = use CV from srv_biom, 1 = yes, 2 = analytically estimate following (Ludwig and Walters 1994)</t>
   </si>
   <si>
-    <t>Sigma_catch_prior</t>
-  </si>
-  <si>
     <t>Starting value to be used if Estimate_sigma_catch = 1</t>
   </si>
   <si>
@@ -399,9 +358,6 @@
     <t>Sel_sd_prior</t>
   </si>
   <si>
-    <t>The sd to use for the random walk of time varying selectivity if set to 1</t>
-  </si>
-  <si>
     <t>Time_varying_q</t>
   </si>
   <si>
@@ -423,21 +379,12 @@
     <t>index to use if catchability coefficients are to be set the same</t>
   </si>
   <si>
-    <t>Sigma_survey_prior</t>
-  </si>
-  <si>
-    <t>Estimate_sigma_survey</t>
-  </si>
-  <si>
     <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
   </si>
   <si>
     <t>Wether a time-varying q should be estimated. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penalty</t>
   </si>
   <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality</t>
-  </si>
-  <si>
     <t>projyr</t>
   </si>
   <si>
@@ -483,13 +430,85 @@
     <t>Sex</t>
   </si>
   <si>
-    <t>sex codes: 0=combined; 1=use female only; 2=use male only</t>
+    <t>fleet_control</t>
+  </si>
+  <si>
+    <t>Fleet_name</t>
+  </si>
+  <si>
+    <t>Fleet_code</t>
+  </si>
+  <si>
+    <t>Name of survey or fishery</t>
+  </si>
+  <si>
+    <t>Index of survey/fishery ACROSS species</t>
+  </si>
+  <si>
+    <t>Fleet_type</t>
+  </si>
+  <si>
+    <t>0 = Do not estimate; 1 = Fishery; 2 = Survey</t>
+  </si>
+  <si>
+    <t>The sd to use for the random walk of time varying selectivity if set to 1. If selectivity is set to type = 2 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>Age_first_selected</t>
+  </si>
+  <si>
+    <t>Age at which selectivity is non-zero</t>
+  </si>
+  <si>
+    <t>Acuumulation_age_lower</t>
+  </si>
+  <si>
+    <t>Ages below this will be grouped to this age for composition data. For example, if set to 2, comp data for age 2 will include 1 and 2 year olds.</t>
+  </si>
+  <si>
+    <t>Acuumulation_age_upper</t>
+  </si>
+  <si>
+    <t>Ages above this will be grouped to this age for composition data. For example, if set to 9 for a species with 10 ages, comp data for age 9 will include 9 and 10 year olds.</t>
+  </si>
+  <si>
+    <t>Log_q_prior</t>
+  </si>
+  <si>
+    <t>Survey_sd_prior</t>
+  </si>
+  <si>
+    <t>Estimate_survey_sd</t>
+  </si>
+  <si>
+    <t>Estimate_catch_sd</t>
+  </si>
+  <si>
+    <t>Catch_sd_prior</t>
+  </si>
+  <si>
+    <t>Comp_weights</t>
+  </si>
+  <si>
+    <t>Composition weights to be used for multinomial likelihood. These are multiplied. After running model, these will update to McAllister &amp; Ianelli 1997 weights using the harmonic mean.</t>
+  </si>
+  <si>
+    <t>proj_F_prop</t>
+  </si>
+  <si>
+    <t>The proportion of future fishing mortality assigned to this fleet</t>
+  </si>
+  <si>
+    <t>sex codes: 0=combined; 1=use female only; 2=use male only; 3 = joint female and male</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1306,40 +1325,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G51"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="119.42578125" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.5" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1350,16 +1369,16 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F2" t="s">
-        <v>86</v>
+        <v>137</v>
       </c>
       <c r="G2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1370,16 +1389,16 @@
         <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>138</v>
       </c>
       <c r="G3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1390,96 +1409,96 @@
         <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F4" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="G4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="G5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F7" t="s">
-        <v>153</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="C8" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G8" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1490,36 +1509,36 @@
         <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F9" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="C10" t="s">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="G10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1530,16 +1549,16 @@
         <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>145</v>
       </c>
       <c r="G11" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1550,36 +1569,36 @@
         <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>60</v>
+        <v>136</v>
       </c>
       <c r="F12" t="s">
-        <v>93</v>
+        <v>147</v>
       </c>
       <c r="G12" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" t="s">
+        <v>136</v>
+      </c>
+      <c r="F13" t="s">
         <v>149</v>
       </c>
-      <c r="C13" t="s">
+      <c r="G13" t="s">
         <v>150</v>
       </c>
-      <c r="D13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F13" t="s">
-        <v>94</v>
-      </c>
-      <c r="G13" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1587,39 +1606,39 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D14" t="s">
+        <v>136</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" t="s">
         <v>103</v>
       </c>
-      <c r="D14" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G14" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>114</v>
+        <v>136</v>
+      </c>
+      <c r="F15" t="s">
+        <v>87</v>
       </c>
       <c r="G15" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1630,16 +1649,16 @@
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
+      </c>
+      <c r="F16" t="s">
+        <v>88</v>
       </c>
       <c r="G16" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1650,16 +1669,16 @@
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
+      </c>
+      <c r="F17" t="s">
+        <v>117</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>10</v>
       </c>
@@ -1670,16 +1689,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>119</v>
+        <v>136</v>
+      </c>
+      <c r="F18" t="s">
+        <v>89</v>
       </c>
       <c r="G18" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>11</v>
       </c>
@@ -1690,16 +1709,16 @@
         <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>121</v>
+        <v>136</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>151</v>
       </c>
       <c r="G19" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>12</v>
       </c>
@@ -1710,16 +1729,16 @@
         <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>11</v>
+        <v>136</v>
       </c>
       <c r="F20" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="G20" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>13</v>
       </c>
@@ -1730,16 +1749,16 @@
         <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="F21" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G21" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>14</v>
       </c>
@@ -1750,16 +1769,16 @@
         <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" t="s">
-        <v>127</v>
+        <v>136</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>153</v>
       </c>
       <c r="G22" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>15</v>
       </c>
@@ -1770,16 +1789,16 @@
         <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" t="s">
-        <v>128</v>
+        <v>136</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>152</v>
       </c>
       <c r="G23" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>16</v>
       </c>
@@ -1790,16 +1809,16 @@
         <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" t="s">
-        <v>130</v>
+        <v>136</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>154</v>
       </c>
       <c r="G24" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>17</v>
       </c>
@@ -1810,16 +1829,16 @@
         <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>16</v>
-      </c>
-      <c r="F25" t="s">
-        <v>132</v>
+        <v>136</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>155</v>
       </c>
       <c r="G25" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>18</v>
       </c>
@@ -1830,10 +1849,16 @@
         <v>57</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G26" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>19</v>
       </c>
@@ -1844,10 +1869,16 @@
         <v>58</v>
       </c>
       <c r="D27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+      <c r="F27" t="s">
+        <v>86</v>
+      </c>
+      <c r="G27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>20</v>
       </c>
@@ -1858,10 +1889,16 @@
         <v>59</v>
       </c>
       <c r="D28" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G28" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>21</v>
       </c>
@@ -1869,16 +1906,10 @@
         <v>20</v>
       </c>
       <c r="C29" t="s">
-        <v>62</v>
-      </c>
-      <c r="D29" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>22</v>
       </c>
@@ -1886,16 +1917,16 @@
         <v>21</v>
       </c>
       <c r="C30" t="s">
-        <v>63</v>
-      </c>
-      <c r="D30" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="F30" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="G30" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>23</v>
       </c>
@@ -1903,16 +1934,10 @@
         <v>22</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D31" t="s">
-        <v>22</v>
-      </c>
-      <c r="F31" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>24</v>
       </c>
@@ -1920,13 +1945,10 @@
         <v>23</v>
       </c>
       <c r="C32" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>25</v>
       </c>
@@ -1934,13 +1956,13 @@
         <v>24</v>
       </c>
       <c r="C33" t="s">
-        <v>66</v>
-      </c>
-      <c r="D33" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+      <c r="F33" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>26</v>
       </c>
@@ -1948,13 +1970,13 @@
         <v>25</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
-      </c>
-      <c r="D34" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="F34" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>27</v>
       </c>
@@ -1962,13 +1984,13 @@
         <v>26</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
-      </c>
-      <c r="D35" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="F35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>28</v>
       </c>
@@ -1976,13 +1998,11 @@
         <v>27</v>
       </c>
       <c r="C36" t="s">
-        <v>106</v>
-      </c>
-      <c r="D36" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>29</v>
       </c>
@@ -1990,13 +2010,10 @@
         <v>28</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
-      </c>
-      <c r="D37" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>30</v>
       </c>
@@ -2004,13 +2021,10 @@
         <v>29</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
-      </c>
-      <c r="D38" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>31</v>
       </c>
@@ -2018,13 +2032,10 @@
         <v>30</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
-      </c>
-      <c r="D39" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>32</v>
       </c>
@@ -2032,13 +2043,10 @@
         <v>31</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
-      </c>
-      <c r="D40" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>33</v>
       </c>
@@ -2046,13 +2054,10 @@
         <v>32</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
-      </c>
-      <c r="D41" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>34</v>
       </c>
@@ -2060,13 +2065,10 @@
         <v>33</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
-      </c>
-      <c r="D42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>35</v>
       </c>
@@ -2074,13 +2076,10 @@
         <v>34</v>
       </c>
       <c r="C43" t="s">
-        <v>72</v>
-      </c>
-      <c r="D43" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>36</v>
       </c>
@@ -2088,13 +2087,10 @@
         <v>35</v>
       </c>
       <c r="C44" t="s">
-        <v>72</v>
-      </c>
-      <c r="D44" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>37</v>
       </c>
@@ -2102,13 +2098,10 @@
         <v>36</v>
       </c>
       <c r="C45" t="s">
-        <v>73</v>
-      </c>
-      <c r="D45" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>38</v>
       </c>
@@ -2116,13 +2109,10 @@
         <v>37</v>
       </c>
       <c r="C46" t="s">
-        <v>74</v>
-      </c>
-      <c r="D46" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>39</v>
       </c>
@@ -2130,66 +2120,51 @@
         <v>38</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
-      </c>
-      <c r="D47" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C48" t="s">
-        <v>82</v>
-      </c>
-      <c r="D48" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>41</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>83</v>
-      </c>
-      <c r="D49" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>42</v>
       </c>
       <c r="B50" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C50" t="s">
-        <v>84</v>
-      </c>
-      <c r="D50" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>43</v>
       </c>
       <c r="B51" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C51" t="s">
-        <v>85</v>
-      </c>
-      <c r="D51" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated ceattle to not bug out for 1 species models
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10810"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grant Adams\Documents\GitHub\Rceattle\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0BF229-F42D-1249-8354-90EAE7EBF434}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="465" windowWidth="25605" windowHeight="12345"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -295,9 +294,6 @@
     <t>Species number</t>
   </si>
   <si>
-    <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic</t>
-  </si>
-  <si>
     <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2. Not used otherwise</t>
   </si>
   <si>
@@ -503,12 +499,15 @@
   </si>
   <si>
     <t>sex codes: 0=combined; 1=use female only; 2=use male only; 3 = joint female and male</t>
+  </si>
+  <si>
+    <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic; 4 = descending logistic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1325,17 +1324,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="119.5" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="119.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -1349,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1369,16 +1368,16 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F2" t="s">
         <v>136</v>
       </c>
-      <c r="F2" t="s">
-        <v>137</v>
-      </c>
       <c r="G2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1389,16 +1388,16 @@
         <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1409,27 +1408,27 @@
         <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F4" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" t="s">
         <v>141</v>
       </c>
-      <c r="G4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C5" t="s">
         <v>121</v>
       </c>
-      <c r="C5" t="s">
-        <v>122</v>
-      </c>
       <c r="D5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F5" t="s">
         <v>83</v>
@@ -1438,67 +1437,67 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" t="s">
         <v>115</v>
       </c>
-      <c r="G6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" t="s">
         <v>124</v>
       </c>
-      <c r="C7" t="s">
-        <v>125</v>
-      </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F7" t="s">
         <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" t="s">
         <v>126</v>
       </c>
-      <c r="C8" t="s">
-        <v>127</v>
-      </c>
       <c r="D8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F8" t="s">
         <v>85</v>
       </c>
       <c r="G8" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1509,36 +1508,36 @@
         <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G9" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" t="s">
         <v>129</v>
       </c>
-      <c r="C10" t="s">
-        <v>130</v>
-      </c>
       <c r="D10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G10" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1549,16 +1548,16 @@
         <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F11" t="s">
+        <v>144</v>
+      </c>
+      <c r="G11" t="s">
         <v>145</v>
       </c>
-      <c r="G11" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1569,36 +1568,36 @@
         <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F12" t="s">
+        <v>146</v>
+      </c>
+      <c r="G12" t="s">
         <v>147</v>
       </c>
-      <c r="G12" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" t="s">
         <v>131</v>
       </c>
-      <c r="C13" t="s">
-        <v>132</v>
-      </c>
       <c r="D13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F13" t="s">
+        <v>148</v>
+      </c>
+      <c r="G13" t="s">
         <v>149</v>
       </c>
-      <c r="G13" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1606,39 +1605,39 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="G14" t="s">
         <v>102</v>
       </c>
-      <c r="G14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" t="s">
         <v>133</v>
       </c>
-      <c r="C15" t="s">
-        <v>134</v>
-      </c>
       <c r="D15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F15" t="s">
         <v>87</v>
       </c>
       <c r="G15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1649,16 +1648,16 @@
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F16" t="s">
         <v>88</v>
       </c>
       <c r="G16" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1669,16 +1668,16 @@
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F17" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" t="s">
         <v>117</v>
       </c>
-      <c r="G17" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>10</v>
       </c>
@@ -1689,16 +1688,16 @@
         <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
       <c r="G18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>11</v>
       </c>
@@ -1709,16 +1708,16 @@
         <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G19" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>12</v>
       </c>
@@ -1729,16 +1728,16 @@
         <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G20" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>13</v>
       </c>
@@ -1749,16 +1748,16 @@
         <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F21" t="s">
+        <v>112</v>
+      </c>
+      <c r="G21" t="s">
         <v>113</v>
       </c>
-      <c r="G21" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>14</v>
       </c>
@@ -1769,16 +1768,16 @@
         <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G22" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>15</v>
       </c>
@@ -1789,16 +1788,16 @@
         <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G23" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>16</v>
       </c>
@@ -1809,16 +1808,16 @@
         <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>17</v>
       </c>
@@ -1829,16 +1828,16 @@
         <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>18</v>
       </c>
@@ -1849,16 +1848,16 @@
         <v>57</v>
       </c>
       <c r="D26" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F26" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G26" t="s">
         <v>156</v>
       </c>
-      <c r="G26" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>19</v>
       </c>
@@ -1869,16 +1868,16 @@
         <v>58</v>
       </c>
       <c r="D27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F27" t="s">
         <v>86</v>
       </c>
       <c r="G27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>20</v>
       </c>
@@ -1889,16 +1888,16 @@
         <v>59</v>
       </c>
       <c r="D28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G28" t="s">
         <v>158</v>
       </c>
-      <c r="G28" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>21</v>
       </c>
@@ -1909,7 +1908,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>22</v>
       </c>
@@ -1920,13 +1919,13 @@
         <v>62</v>
       </c>
       <c r="F30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G30" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>23</v>
       </c>
@@ -1937,7 +1936,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>24</v>
       </c>
@@ -1948,7 +1947,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>25</v>
       </c>
@@ -1959,10 +1958,10 @@
         <v>65</v>
       </c>
       <c r="F33" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>26</v>
       </c>
@@ -1973,10 +1972,10 @@
         <v>73</v>
       </c>
       <c r="F34" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>27</v>
       </c>
@@ -1987,10 +1986,10 @@
         <v>67</v>
       </c>
       <c r="F35" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>28</v>
       </c>
@@ -1998,11 +1997,11 @@
         <v>27</v>
       </c>
       <c r="C36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>29</v>
       </c>
@@ -2013,7 +2012,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>30</v>
       </c>
@@ -2024,7 +2023,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>31</v>
       </c>
@@ -2035,7 +2034,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>32</v>
       </c>
@@ -2046,7 +2045,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>33</v>
       </c>
@@ -2057,7 +2056,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>34</v>
       </c>
@@ -2068,7 +2067,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>35</v>
       </c>
@@ -2079,7 +2078,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>36</v>
       </c>
@@ -2090,7 +2089,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>37</v>
       </c>
@@ -2101,7 +2100,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>38</v>
       </c>
@@ -2112,7 +2111,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>39</v>
       </c>
@@ -2123,7 +2122,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>40</v>
       </c>
@@ -2134,7 +2133,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>41</v>
       </c>
@@ -2145,7 +2144,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>42</v>
       </c>
@@ -2156,7 +2155,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Martin's Likes, Analytical q change, Q prior
Added martin's likelihoods to cpp
Updated analytical q to account for time varying sigma as input by user
Changed q selection to have a prior on q
1 = est param, 2 = est param with prior, 3 = analytical, 4 = power function
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -450,9 +450,6 @@
     <t>The sd to use for the random walk of time varying selectivity if set to 1. If selectivity is set to type = 2 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
   </si>
   <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penality. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
-  </si>
-  <si>
     <t>Age_first_selected</t>
   </si>
   <si>
@@ -502,6 +499,9 @@
   </si>
   <si>
     <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic; 4 = descending logistic</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity, or descending logistic. 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
   </si>
 </sst>
 </file>
@@ -1474,7 +1474,7 @@
         <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1514,7 +1514,7 @@
         <v>109</v>
       </c>
       <c r="G9" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1551,10 +1551,10 @@
         <v>135</v>
       </c>
       <c r="F11" t="s">
+        <v>143</v>
+      </c>
+      <c r="G11" t="s">
         <v>144</v>
-      </c>
-      <c r="G11" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1571,10 +1571,10 @@
         <v>135</v>
       </c>
       <c r="F12" t="s">
+        <v>145</v>
+      </c>
+      <c r="G12" t="s">
         <v>146</v>
-      </c>
-      <c r="G12" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1591,10 +1591,10 @@
         <v>135</v>
       </c>
       <c r="F13" t="s">
+        <v>147</v>
+      </c>
+      <c r="G13" t="s">
         <v>148</v>
-      </c>
-      <c r="G13" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1711,7 +1711,7 @@
         <v>135</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G19" t="s">
         <v>96</v>
@@ -1771,7 +1771,7 @@
         <v>135</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G22" t="s">
         <v>104</v>
@@ -1791,7 +1791,7 @@
         <v>135</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G23" t="s">
         <v>105</v>
@@ -1811,7 +1811,7 @@
         <v>135</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G24" t="s">
         <v>106</v>
@@ -1831,7 +1831,7 @@
         <v>135</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G25" t="s">
         <v>107</v>
@@ -1851,10 +1851,10 @@
         <v>135</v>
       </c>
       <c r="F26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G26" t="s">
         <v>155</v>
-      </c>
-      <c r="G26" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1891,10 +1891,10 @@
         <v>135</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G28" t="s">
         <v>157</v>
-      </c>
-      <c r="G28" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1922,7 +1922,7 @@
         <v>134</v>
       </c>
       <c r="G30" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added sex ratio to likelihood, changed propF to sex_ratio
For two sex models, added sex ratio to the model likelihood. The use inputs the mean in the sex_ratio data and the variance in the control. est_sex_ratio = 0, does not estimate; 1 = estimate using annual mean across ages (uses age2 in sex_ratio), 2 = estimate using annual and age specific estimates.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="160">
   <si>
     <t>nspp</t>
   </si>
@@ -48,30 +48,18 @@
     <t>stom_sample_size</t>
   </si>
   <si>
-    <t>srv_control</t>
-  </si>
-  <si>
     <t>srv_biom</t>
   </si>
   <si>
     <t>srv_emp_sel</t>
   </si>
   <si>
-    <t>srv_comp</t>
-  </si>
-  <si>
-    <t>fsh_control</t>
-  </si>
-  <si>
     <t>fsh_biom</t>
   </si>
   <si>
     <t>fsh_emp_sel</t>
   </si>
   <si>
-    <t>fsh_comp</t>
-  </si>
-  <si>
     <t>age_trans_matrix</t>
   </si>
   <si>
@@ -168,18 +156,9 @@
     <t>Sample size of diet data for each species (used when suitMode &gt; 0)</t>
   </si>
   <si>
-    <t>Survey data specifications</t>
-  </si>
-  <si>
     <t>Empirical selectivity for surveys (leave empty if not used)</t>
   </si>
   <si>
-    <t>Survey age or length composition data</t>
-  </si>
-  <si>
-    <t>Fishery data specifications</t>
-  </si>
-  <si>
     <t>Total catch in weight (kg) or numbers data</t>
   </si>
   <si>
@@ -189,9 +168,6 @@
     <t>Empirical selectivity for fisheries (leave empty if not used)</t>
   </si>
   <si>
-    <t>Fishery age or length composition data</t>
-  </si>
-  <si>
     <t>Age transition matrix (e.g. Age Length Key or ALK) used to convert age to length for length comp data. Can have multiple ALKs for a species specified by ALK_index.</t>
   </si>
   <si>
@@ -502,6 +478,27 @@
   </si>
   <si>
     <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity, or descending logistic. 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>Survey and fishery data specifications</t>
+  </si>
+  <si>
+    <t>comp</t>
+  </si>
+  <si>
+    <t>Survey/fishery age or length composition data</t>
+  </si>
+  <si>
+    <t>est_propF</t>
+  </si>
+  <si>
+    <t>propF_sigma</t>
+  </si>
+  <si>
+    <t>Is sex ration F/(M+F) to be included in the likelihood (assumed normal); 0 = no, 1 = use annual average across ages (uses 2nd age in propF data), 2 = age, and year specific (TBD)</t>
+  </si>
+  <si>
+    <t>Initial value or fixed value for sd of normal likelihood for sex ration. Not yet able to estimate.</t>
   </si>
 </sst>
 </file>
@@ -1336,25 +1333,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1365,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F2" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="G2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1385,16 +1382,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F3" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="G3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1405,16 +1402,16 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F4" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="G4" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1422,19 +1419,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C5" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D5" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F5" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="G5" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1442,19 +1439,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D6" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F6" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="G6" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1462,19 +1459,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C7" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D7" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F7" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="G7" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1482,19 +1479,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D8" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F8" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G8" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1505,16 +1502,16 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F9" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="G9" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1522,19 +1519,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D10" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F10" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="G10" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1545,16 +1542,16 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
+        <v>127</v>
+      </c>
+      <c r="F11" t="s">
         <v>135</v>
       </c>
-      <c r="F11" t="s">
-        <v>143</v>
-      </c>
       <c r="G11" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1565,16 +1562,16 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F12" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="G12" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1582,19 +1579,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C13" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D13" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="G13" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1605,16 +1602,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" t="s">
+        <v>127</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" t="s">
         <v>94</v>
-      </c>
-      <c r="D14" t="s">
-        <v>135</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="G14" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1622,19 +1619,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C15" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D15" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1645,16 +1642,16 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D16" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G16" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1665,16 +1662,16 @@
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D17" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F17" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="G17" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1682,19 +1679,19 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="D18" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F18" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="G18" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1702,19 +1699,19 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>10</v>
+        <v>157</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>159</v>
       </c>
       <c r="D19" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="G19" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1722,19 +1719,19 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>127</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>153</v>
       </c>
       <c r="D20" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F20" t="s">
+        <v>103</v>
+      </c>
+      <c r="G20" t="s">
         <v>111</v>
-      </c>
-      <c r="G20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1742,19 +1739,19 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D21" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F21" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="G21" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1762,19 +1759,19 @@
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D22" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="G22" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1782,19 +1779,19 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>154</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>155</v>
       </c>
       <c r="D23" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="G23" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1802,19 +1799,19 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="D24" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="G24" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1822,19 +1819,19 @@
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="G25" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1842,19 +1839,19 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D26" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="G26" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1862,19 +1859,19 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="G27" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1882,19 +1879,19 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D28" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="G28" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1902,10 +1899,10 @@
         <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1913,16 +1910,16 @@
         <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C30" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="F30" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G30" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1930,10 +1927,10 @@
         <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1941,10 +1938,10 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C32" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1952,13 +1949,13 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F33" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1966,13 +1963,13 @@
         <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C34" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F34" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1980,13 +1977,13 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F35" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1994,10 +1991,10 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C36" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="F36" s="4"/>
     </row>
@@ -2006,10 +2003,10 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C37" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2017,10 +2014,10 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C38" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2028,10 +2025,10 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C39" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2039,10 +2036,10 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2050,10 +2047,10 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C41" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2061,10 +2058,10 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C42" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2072,10 +2069,10 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C43" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2083,10 +2080,10 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2094,10 +2091,10 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C45" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2105,10 +2102,10 @@
         <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C46" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2116,10 +2113,10 @@
         <v>39</v>
       </c>
       <c r="B47" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C47" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2127,10 +2124,10 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C48" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -2138,10 +2135,10 @@
         <v>41</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C49" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -2149,10 +2146,10 @@
         <v>42</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -2160,10 +2157,10 @@
         <v>43</v>
       </c>
       <c r="B51" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C51" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Allowed multiple environmental indices and environmentally driven q
Allowed for multiple environmental indices by changing BTemp to env_data and inputting as matrix
Bioenegetics is driven by the index selected by Cindex
Added Estimate_q = 5, where catchability ln(q_y) = q_mu + beta * index_y. Where the index is selected by the Time_varying_q column in fleet control
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="162">
   <si>
     <t>nspp</t>
   </si>
@@ -117,12 +117,6 @@
     <t>CK4</t>
   </si>
   <si>
-    <t>Tyrs</t>
-  </si>
-  <si>
-    <t>BTempC</t>
-  </si>
-  <si>
     <t>Pyrs</t>
   </si>
   <si>
@@ -210,12 +204,6 @@
     <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
   </si>
   <si>
-    <t xml:space="preserve">Years of bottom temperature data to incorporate into ft specificed by Ceq. </t>
-  </si>
-  <si>
-    <t>Bottom temperature data to incorporate into ft specificed by Ceq. Will use the mean for missing years.</t>
-  </si>
-  <si>
     <t>Which bioenergetics equation to use for each species for ft to scale max consumtion: 1 = Exponential (Stewart et al 1983), 2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015), 3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979)</t>
   </si>
   <si>
@@ -306,9 +294,6 @@
     <t>Is the observation in weight (kg) set as 1, if the observation is in numbers caught, set as 2</t>
   </si>
   <si>
-    <t>Estimate catchability? (0 = no; 1 = yes, 2 = analytical from Ludwig and Walters 1994)</t>
-  </si>
-  <si>
     <t>Estimate survey variance (0 = use CV from srv_biom, 1 = yes, 2 = analytically estimate following (Ludwig and Walters 1994)</t>
   </si>
   <si>
@@ -354,9 +339,6 @@
     <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
   </si>
   <si>
-    <t>Wether a time-varying q should be estimated. 0 = no, 1 = random walk from mean selectivity following Dorn 2018, 2 = random effect, 3 = time blocks with no penalty</t>
-  </si>
-  <si>
     <t>projyr</t>
   </si>
   <si>
@@ -444,9 +426,6 @@
     <t>Ages above this will be grouped to this age for composition data. For example, if set to 9 for a species with 10 ages, comp data for age 9 will include 9 and 10 year olds.</t>
   </si>
   <si>
-    <t>Log_q_prior</t>
-  </si>
-  <si>
     <t>Survey_sd_prior</t>
   </si>
   <si>
@@ -477,9 +456,6 @@
     <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic; 4 = descending logistic</t>
   </si>
   <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity, or descending logistic. 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
-  </si>
-  <si>
     <t>Survey and fishery data specifications</t>
   </si>
   <si>
@@ -499,6 +475,36 @@
   </si>
   <si>
     <t>Initial value or fixed value for sd of normal likelihood for sex ration. Not yet able to estimate.</t>
+  </si>
+  <si>
+    <t>Q_prior</t>
+  </si>
+  <si>
+    <t>Time_varying_q_sd_prior</t>
+  </si>
+  <si>
+    <t>Variance of q prior: dnorm (log_q, log_q_prior, q_sd_prior)</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity, or descending logistic. 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic only. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>Wether a time-varying q should be estimated. 0 = no, 1 = penalized deviate, 2 = random effect, 3 = time blocks with no penalty; 4 = random walk from mean following Dorn 2018 (dnorm(q_y - q_y-1, 0, sigma). If Estimate_q = 5, this determines the environmental index to be used in the equation log(q_y) = q_mu + beta * index_y</t>
+  </si>
+  <si>
+    <t>Estimate catchability? (0 = fixed at prior; - 1 = Estimate single parameter; - 2 = Estimate single parameter with prior; - 3 = Estimate analytical q  from Ludwig and Walters 1994;  - 4 = Estimate power equation; - 5 - Linear equation log(q_y) = q_mu + beta * index_y)</t>
+  </si>
+  <si>
+    <t>Cindex</t>
+  </si>
+  <si>
+    <t>Which environmental index in env_data to use to drive bioenergetics</t>
+  </si>
+  <si>
+    <t>env_data</t>
+  </si>
+  <si>
+    <t>Environmental indices such as bottom temperature data to incorporate into ration equation specificed by Ceq and Cindex. Also used to drive catchability if Estimate_q = 5. Will use the mean for missing years. Temperature should be in celcius.</t>
   </si>
 </sst>
 </file>
@@ -1333,25 +1339,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1362,16 +1368,16 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1382,16 +1388,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1402,16 +1408,16 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F4" t="s">
+        <v>126</v>
+      </c>
+      <c r="G4" t="s">
         <v>127</v>
-      </c>
-      <c r="F4" t="s">
-        <v>132</v>
-      </c>
-      <c r="G4" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1419,19 +1425,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1439,19 +1445,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F6" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G6" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1459,19 +1465,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C7" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D7" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F7" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G7" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1479,19 +1485,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D8" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G8" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1502,16 +1508,16 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F9" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="G9" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1519,19 +1525,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D10" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F10" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G10" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1542,16 +1548,16 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F11" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="G11" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1562,16 +1568,16 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F12" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G12" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1579,19 +1585,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C13" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D13" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F13" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="G13" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1602,16 +1608,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D14" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1619,19 +1625,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C15" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D15" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1642,16 +1648,16 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F16" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G16" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1662,16 +1668,16 @@
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="G17" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1679,19 +1685,19 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C18" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D18" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s">
-        <v>95</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1699,19 +1705,19 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C19" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D19" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G19" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1719,19 +1725,19 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C20" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="D20" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F20" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G20" t="s">
-        <v>111</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1742,16 +1748,16 @@
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F21" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="G21" t="s">
-        <v>105</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1762,16 +1768,16 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D22" t="s">
-        <v>127</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>143</v>
+        <v>121</v>
+      </c>
+      <c r="F22" t="s">
+        <v>153</v>
       </c>
       <c r="G22" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1779,19 +1785,19 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C23" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>142</v>
+        <v>121</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>136</v>
       </c>
       <c r="G23" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1802,16 +1808,16 @@
         <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>127</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>144</v>
+        <v>121</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>135</v>
       </c>
       <c r="G24" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1822,16 +1828,16 @@
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
-        <v>127</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>145</v>
+        <v>121</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="G25" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1842,16 +1848,16 @@
         <v>13</v>
       </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D26" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G26" t="s">
-        <v>147</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1862,16 +1868,16 @@
         <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D27" t="s">
-        <v>127</v>
-      </c>
-      <c r="F27" t="s">
-        <v>78</v>
+        <v>121</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>139</v>
       </c>
       <c r="G27" t="s">
-        <v>84</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1882,16 +1888,16 @@
         <v>15</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D28" t="s">
-        <v>127</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>148</v>
+        <v>121</v>
+      </c>
+      <c r="F28" t="s">
+        <v>74</v>
       </c>
       <c r="G28" t="s">
-        <v>149</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1902,7 +1908,13 @@
         <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>51</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G29" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1913,13 +1925,13 @@
         <v>17</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F30" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="G30" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1930,7 +1942,7 @@
         <v>18</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1941,7 +1953,7 @@
         <v>19</v>
       </c>
       <c r="C32" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1952,10 +1964,10 @@
         <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F33" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1966,10 +1978,10 @@
         <v>21</v>
       </c>
       <c r="C34" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F34" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1977,13 +1989,13 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>22</v>
+        <v>158</v>
       </c>
       <c r="C35" t="s">
-        <v>59</v>
+        <v>159</v>
       </c>
       <c r="F35" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1991,33 +2003,33 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C36" t="s">
-        <v>89</v>
-      </c>
-      <c r="F36" s="4"/>
+        <v>57</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
-        <v>60</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C38" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2025,10 +2037,10 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C39" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2036,10 +2048,10 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2047,10 +2059,10 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2058,10 +2070,10 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C42" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2069,10 +2081,10 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C43" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2080,10 +2092,10 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2091,10 +2103,10 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C45" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2102,10 +2114,10 @@
         <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>33</v>
+        <v>160</v>
       </c>
       <c r="C46" t="s">
-        <v>64</v>
+        <v>161</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2113,10 +2125,10 @@
         <v>39</v>
       </c>
       <c r="B47" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C47" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2124,10 +2136,10 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
         <v>67</v>
-      </c>
-      <c r="C48" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -2135,10 +2147,10 @@
         <v>41</v>
       </c>
       <c r="B49" t="s">
+        <v>64</v>
+      </c>
+      <c r="C49" t="s">
         <v>68</v>
-      </c>
-      <c r="C49" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -2146,10 +2158,10 @@
         <v>42</v>
       </c>
       <c r="B50" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" t="s">
         <v>69</v>
-      </c>
-      <c r="C50" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -2157,10 +2169,10 @@
         <v>43</v>
       </c>
       <c r="B51" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" t="s">
         <v>70</v>
-      </c>
-      <c r="C51" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated meta_names in excel, added optimization control to fit mod
Added optimization control to fit_mod and phaser
F now is zero for non-fisheries. Was previously unused for surveys but set at the initial parameter values that were not estimated. Now set to zero.
Removed the environmental q bit in the cpp file because it was giving the cod model some trouble.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="156">
   <si>
     <t>nspp</t>
   </si>
@@ -51,15 +51,9 @@
     <t>srv_biom</t>
   </si>
   <si>
-    <t>srv_emp_sel</t>
-  </si>
-  <si>
     <t>fsh_biom</t>
   </si>
   <si>
-    <t>fsh_emp_sel</t>
-  </si>
-  <si>
     <t>age_trans_matrix</t>
   </si>
   <si>
@@ -150,18 +144,12 @@
     <t>Sample size of diet data for each species (used when suitMode &gt; 0)</t>
   </si>
   <si>
-    <t>Empirical selectivity for surveys (leave empty if not used)</t>
-  </si>
-  <si>
     <t>Total catch in weight (kg) or numbers data</t>
   </si>
   <si>
     <t>Survey index in weight (kg) or numbers data</t>
   </si>
   <si>
-    <t>Empirical selectivity for fisheries (leave empty if not used)</t>
-  </si>
-  <si>
     <t>Age transition matrix (e.g. Age Length Key or ALK) used to convert age to length for length comp data. Can have multiple ALKs for a species specified by ALK_index.</t>
   </si>
   <si>
@@ -189,12 +177,6 @@
     <t>Parameters for weight-at-length power function for each species. . Used when estimating time-variant length-based gamma suitability (suitMode = 2) or time-variant length-based lognormal suitability (suitMode = 5)</t>
   </si>
   <si>
-    <t>data_list Object name</t>
-  </si>
-  <si>
-    <t>This scales the maximum consumption used for ration for each species; Pvalue is in Cmax*fT*Pvalue*Page</t>
-  </si>
-  <si>
     <t>Intercept of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
   </si>
   <si>
@@ -207,33 +189,18 @@
     <t>Which bioenergetics equation to use for each species for ft to scale max consumtion: 1 = Exponential (Stewart et al 1983), 2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015), 3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979)</t>
   </si>
   <si>
-    <t>Annual relative foraging rate by age</t>
-  </si>
-  <si>
     <t>UobsAge</t>
   </si>
   <si>
     <t>UobsWtAge</t>
   </si>
   <si>
-    <t>Uobs</t>
-  </si>
-  <si>
-    <t>UobsWt</t>
-  </si>
-  <si>
     <t>Stomach proportion by numbers for each predator, prey, predator age, prey age combination. Can also be year specific by including the column, "Year"</t>
   </si>
   <si>
     <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Can also be year specific by including the column, "Year"</t>
   </si>
   <si>
-    <t>Stomach proportion by numbers for each predator, prey, predator length, prey length combination. Can also be year specific by including the column, "Year"</t>
-  </si>
-  <si>
-    <t>Stomach proportion by weight for each predator, prey, predator length prey length combination. Can also be year specific by including the column, "Year"</t>
-  </si>
-  <si>
     <t>Species</t>
   </si>
   <si>
@@ -276,9 +243,6 @@
     <t>Starting value or fixed value for catchability</t>
   </si>
   <si>
-    <t>Percent of foraging days per year for each species</t>
-  </si>
-  <si>
     <t>Blank</t>
   </si>
   <si>
@@ -327,9 +291,6 @@
     <t>Selectivity_index</t>
   </si>
   <si>
-    <t>index to use if selectivitys of different surveys are to be the same</t>
-  </si>
-  <si>
     <t>Q_index</t>
   </si>
   <si>
@@ -459,12 +420,6 @@
     <t>Survey and fishery data specifications</t>
   </si>
   <si>
-    <t>comp</t>
-  </si>
-  <si>
-    <t>Survey/fishery age or length composition data</t>
-  </si>
-  <si>
     <t>est_propF</t>
   </si>
   <si>
@@ -505,6 +460,33 @@
   </si>
   <si>
     <t>Environmental indices such as bottom temperature data to incorporate into ration equation specificed by Ceq and Cindex. Also used to drive catchability if Estimate_q = 5. Will use the mean for missing years. Temperature should be in celcius.</t>
+  </si>
+  <si>
+    <t>emp_sel</t>
+  </si>
+  <si>
+    <t>Empirical/fixed selectivity for surveys and fisheries (leave empty if not used)</t>
+  </si>
+  <si>
+    <t>comp_data</t>
+  </si>
+  <si>
+    <t>Survey/fishery age or length composition data. Note if sex is 3, put female composition data then male composition data (similar to SS).</t>
+  </si>
+  <si>
+    <t>Object name</t>
+  </si>
+  <si>
+    <t>index to use if selectivities of different surveys are to be the same</t>
+  </si>
+  <si>
+    <t>Number of foraging days per year for each species</t>
+  </si>
+  <si>
+    <t>This scales the maximum consumption used for ration for each species; Pvalue is in Cmax*fT*Pvalue*Pyrs</t>
+  </si>
+  <si>
+    <t>Annual relative foraging rate by age. Multiplied by pvalue and fday to scale maximum consumption to the number of days in a year that foraging occurs.</t>
   </si>
 </sst>
 </file>
@@ -1328,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -1339,25 +1321,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>151</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1368,16 +1350,16 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F2" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="G2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1388,16 +1370,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F3" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="G3" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1408,16 +1390,16 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="G4" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1425,19 +1407,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1445,19 +1427,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="G6" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1465,19 +1447,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G7" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1485,19 +1467,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="G8" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1508,16 +1490,16 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F9" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G9" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1525,19 +1507,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="C10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" t="s">
         <v>115</v>
-      </c>
-      <c r="D10" t="s">
-        <v>121</v>
-      </c>
-      <c r="F10" t="s">
-        <v>97</v>
-      </c>
-      <c r="G10" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1548,16 +1530,16 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F11" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="G11" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1568,16 +1550,16 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F12" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="G12" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1585,19 +1567,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="C13" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="D13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" t="s">
+        <v>120</v>
+      </c>
+      <c r="G13" t="s">
         <v>121</v>
-      </c>
-      <c r="F13" t="s">
-        <v>133</v>
-      </c>
-      <c r="G13" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1608,16 +1590,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="G14" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1625,19 +1607,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="C15" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F15" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="G15" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1648,16 +1630,16 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F16" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="G16" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1668,16 +1650,16 @@
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="G17" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1685,19 +1667,19 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="C18" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="D18" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F18" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G18" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1705,19 +1687,19 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="C19" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="G19" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1725,19 +1707,19 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="C20" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="D20" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F20" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G20" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1748,16 +1730,16 @@
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F21" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="G21" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1768,16 +1750,16 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D22" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F22" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="G22" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1785,19 +1767,19 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C23" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D23" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="G23" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1805,19 +1787,19 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>147</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
+        <v>148</v>
       </c>
       <c r="D24" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="G24" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1825,19 +1807,19 @@
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D25" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="G25" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1845,19 +1827,19 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="G26" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1865,19 +1847,19 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C27" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D27" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="G27" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1885,19 +1867,19 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F28" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="G28" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1905,16 +1887,16 @@
         <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="G29" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1922,16 +1904,16 @@
         <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F30" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="G30" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1939,10 +1921,10 @@
         <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C31" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1950,10 +1932,10 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1961,13 +1943,13 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C33" t="s">
         <v>55</v>
       </c>
       <c r="F33" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1975,13 +1957,13 @@
         <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>21</v>
+        <v>143</v>
       </c>
       <c r="C34" t="s">
-        <v>61</v>
+        <v>144</v>
       </c>
       <c r="F34" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1989,13 +1971,13 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>158</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F35" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2003,10 +1985,10 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C36" t="s">
-        <v>57</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2014,10 +1996,10 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C37" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="F37" s="4"/>
     </row>
@@ -2026,10 +2008,10 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C38" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2037,10 +2019,10 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C39" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2048,10 +2030,10 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C40" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2059,10 +2041,10 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2070,10 +2052,10 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C42" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2081,10 +2063,10 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C43" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2092,10 +2074,10 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C44" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2103,10 +2085,10 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>31</v>
+        <v>145</v>
       </c>
       <c r="C45" t="s">
-        <v>60</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2114,10 +2096,10 @@
         <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>160</v>
+        <v>30</v>
       </c>
       <c r="C46" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2125,10 +2107,10 @@
         <v>39</v>
       </c>
       <c r="B47" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C47" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2136,43 +2118,10 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C48" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>41</v>
-      </c>
-      <c r="B49" t="s">
-        <v>64</v>
-      </c>
-      <c r="C49" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>42</v>
-      </c>
-      <c r="B50" t="s">
-        <v>65</v>
-      </c>
-      <c r="C50" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>43</v>
-      </c>
-      <c r="B51" t="s">
-        <v>66</v>
-      </c>
-      <c r="C51" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Renamed ALK to Age_transition where appropriate
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -39,9 +39,6 @@
     <t>pop_wt_index</t>
   </si>
   <si>
-    <t>pop_alk_index</t>
-  </si>
-  <si>
     <t>other_food</t>
   </si>
   <si>
@@ -150,9 +147,6 @@
     <t>Survey index in weight (kg) or numbers data</t>
   </si>
   <si>
-    <t>Age transition matrix (e.g. Age Length Key or ALK) used to convert age to length for length comp data. Can have multiple ALKs for a species specified by ALK_index.</t>
-  </si>
-  <si>
     <t>Aging error matrices. Can have only one per species.</t>
   </si>
   <si>
@@ -216,9 +210,6 @@
     <t>Weight_index</t>
   </si>
   <si>
-    <t>ALK_index</t>
-  </si>
-  <si>
     <t>Estimate_q</t>
   </si>
   <si>
@@ -234,12 +225,6 @@
     <t>Weight-at-age (wt) index to use for calculation of derived quantities</t>
   </si>
   <si>
-    <t>Age transition matrix (e.g. Age Length Key or ALK) index to use for derived quantities of the population (used in length-based predation estimation)</t>
-  </si>
-  <si>
-    <t>Age transition matrix (e.g. Age Length Key or ALK) index to use for derived quantitied</t>
-  </si>
-  <si>
     <t>Starting value or fixed value for catchability</t>
   </si>
   <si>
@@ -487,6 +472,21 @@
   </si>
   <si>
     <t>Annual relative foraging rate by age. Multiplied by pvalue and fday to scale maximum consumption to the number of days in a year that foraging occurs.</t>
+  </si>
+  <si>
+    <t>pop_age_transition_index</t>
+  </si>
+  <si>
+    <t>Age transition matrix (e.g. growth trajectory) index to use for derived quantities of the population to convert age to length (also used in length-based predation estimation)</t>
+  </si>
+  <si>
+    <t>Age_transition_index</t>
+  </si>
+  <si>
+    <t>Age transition matrix (e.g. growth trajectory) index to use for derived quantities to convert age to length</t>
+  </si>
+  <si>
+    <t>Age transition matrix (e.g. growth trajectory) used to convert age to length for length comp data. Can have multiple matrices for a species specified by Age_transition_index.</t>
   </si>
 </sst>
 </file>
@@ -1321,25 +1321,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1350,16 +1350,16 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="G2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1370,16 +1370,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="G3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1390,16 +1390,16 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" t="s">
         <v>108</v>
       </c>
-      <c r="F4" t="s">
-        <v>113</v>
-      </c>
       <c r="G4" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1407,19 +1407,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1427,19 +1427,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" t="s">
         <v>95</v>
       </c>
-      <c r="C6" t="s">
-        <v>100</v>
-      </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G6" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1447,19 +1447,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G7" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1467,19 +1467,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1490,16 +1490,16 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F9" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G9" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1507,19 +1507,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1530,16 +1530,16 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F11" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G11" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1550,16 +1550,16 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F12" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G12" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1567,19 +1567,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F13" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1587,19 +1587,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>6</v>
+        <v>151</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>152</v>
       </c>
       <c r="D14" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1607,19 +1607,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D15" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1627,19 +1627,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>153</v>
       </c>
       <c r="G16" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1647,19 +1647,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F17" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1667,19 +1667,19 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D18" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G18" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1687,19 +1687,19 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C19" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D19" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1707,19 +1707,19 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D20" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F20" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G20" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1727,19 +1727,19 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F21" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1747,19 +1747,19 @@
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D22" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G22" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1767,19 +1767,19 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G23" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1787,19 +1787,19 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C24" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D24" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="G24" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1807,19 +1807,19 @@
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>43</v>
+        <v>155</v>
       </c>
       <c r="D25" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G25" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1827,19 +1827,19 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="G26" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1847,19 +1847,19 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D27" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G27" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1867,19 +1867,19 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D28" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1887,16 +1887,16 @@
         <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G29" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1904,16 +1904,16 @@
         <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F30" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G30" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1921,10 +1921,10 @@
         <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1932,10 +1932,10 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C32" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1943,13 +1943,13 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F33" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1957,13 +1957,13 @@
         <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C34" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="F34" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1971,13 +1971,13 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="F35" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1985,10 +1985,10 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1996,10 +1996,10 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F37" s="4"/>
     </row>
@@ -2008,10 +2008,10 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2019,10 +2019,10 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2030,10 +2030,10 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2041,10 +2041,10 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C41" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2052,10 +2052,10 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C42" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2063,10 +2063,10 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C43" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2074,10 +2074,10 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C44" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2085,10 +2085,10 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C45" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2096,10 +2096,10 @@
         <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C46" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2107,10 +2107,10 @@
         <v>39</v>
       </c>
       <c r="B47" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" t="s">
         <v>56</v>
-      </c>
-      <c r="C47" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2118,10 +2118,10 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" t="s">
         <v>57</v>
-      </c>
-      <c r="C48" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed some old files and updated roxygen for data and fixed age_trans name bug from last commit
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="156">
   <si>
     <t>nspp</t>
   </si>
@@ -1892,6 +1892,9 @@
       <c r="C29" t="s">
         <v>46</v>
       </c>
+      <c r="D29" t="s">
+        <v>103</v>
+      </c>
       <c r="F29" s="2" t="s">
         <v>123</v>
       </c>

</xml_diff>

<commit_message>
Fixed plot_logindex and debugged non-parametric sel
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -345,9 +345,6 @@
     <t>sex codes: 0=combined; 1=use female only; 2=use male only; 3 = joint female and male</t>
   </si>
   <si>
-    <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic; 4 = descending logistic</t>
-  </si>
-  <si>
     <t>Survey and fishery data specifications</t>
   </si>
   <si>
@@ -502,6 +499,9 @@
   </si>
   <si>
     <t>Numeric: number of foraging days per year for each species</t>
+  </si>
+  <si>
+    <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic; 4 = descending logistic; 5 = non-parametric selectivity sensu Taylor et al 2014 (Hake)</t>
   </si>
 </sst>
 </file>
@@ -1343,7 +1343,7 @@
         <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>30</v>
@@ -1363,13 +1363,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E2" t="s">
         <v>85</v>
@@ -1386,13 +1386,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E3" t="s">
         <v>85</v>
@@ -1409,13 +1409,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E4" t="s">
         <v>85</v>
@@ -1432,13 +1432,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C5" t="s">
         <v>77</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E5" t="s">
         <v>85</v>
@@ -1455,13 +1455,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" t="s">
         <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E6" t="s">
         <v>85</v>
@@ -1470,7 +1470,7 @@
         <v>73</v>
       </c>
       <c r="G6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1478,13 +1478,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C7" t="s">
         <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E7" t="s">
         <v>85</v>
@@ -1493,7 +1493,7 @@
         <v>49</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1501,13 +1501,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C8" t="s">
         <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E8" t="s">
         <v>85</v>
@@ -1524,13 +1524,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E9" t="s">
         <v>85</v>
@@ -1539,7 +1539,7 @@
         <v>68</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1547,13 +1547,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C10" t="s">
         <v>81</v>
       </c>
       <c r="D10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E10" t="s">
         <v>85</v>
@@ -1570,13 +1570,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C11" t="s">
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E11" t="s">
         <v>85</v>
@@ -1593,13 +1593,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E12" t="s">
         <v>85</v>
@@ -1616,13 +1616,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C13" t="s">
         <v>82</v>
       </c>
       <c r="D13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E13" t="s">
         <v>85</v>
@@ -1639,13 +1639,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E14" t="s">
         <v>85</v>
@@ -1662,13 +1662,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C15" t="s">
         <v>83</v>
       </c>
       <c r="D15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E15" t="s">
         <v>85</v>
@@ -1685,22 +1685,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E16" t="s">
         <v>85</v>
       </c>
       <c r="F16" t="s">
+        <v>126</v>
+      </c>
+      <c r="G16" t="s">
         <v>127</v>
-      </c>
-      <c r="G16" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1708,13 +1708,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E17" t="s">
         <v>85</v>
@@ -1731,13 +1731,13 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C18" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" t="s">
         <v>134</v>
-      </c>
-      <c r="D18" t="s">
-        <v>135</v>
       </c>
       <c r="E18" t="s">
         <v>85</v>
@@ -1746,7 +1746,7 @@
         <v>53</v>
       </c>
       <c r="G18" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1754,19 +1754,19 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E19" t="s">
         <v>85</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G19" t="s">
         <v>58</v>
@@ -1777,13 +1777,13 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D20" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E20" t="s">
         <v>85</v>
@@ -1792,7 +1792,7 @@
         <v>71</v>
       </c>
       <c r="G20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1800,13 +1800,13 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D21" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E21" t="s">
         <v>85</v>
@@ -1815,7 +1815,7 @@
         <v>70</v>
       </c>
       <c r="G21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1826,13 +1826,13 @@
         <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E22" t="s">
         <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G22" t="s">
         <v>72</v>
@@ -1883,10 +1883,10 @@
         <v>17</v>
       </c>
       <c r="C25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" t="s">
         <v>121</v>
-      </c>
-      <c r="D25" t="s">
-        <v>122</v>
       </c>
       <c r="E25" t="s">
         <v>85</v>
@@ -1903,10 +1903,10 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" t="s">
         <v>119</v>
-      </c>
-      <c r="D26" t="s">
-        <v>120</v>
       </c>
       <c r="E26" t="s">
         <v>85</v>
@@ -1926,7 +1926,7 @@
         <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E27" t="s">
         <v>85</v>
@@ -2050,13 +2050,13 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
       </c>
       <c r="D35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F35" t="s">
         <v>76</v>
@@ -2067,13 +2067,13 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C36" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2081,13 +2081,13 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C37" t="s">
         <v>18</v>
       </c>
       <c r="D37" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F37" s="4"/>
     </row>
@@ -2096,13 +2096,13 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2110,7 +2110,7 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C39" t="s">
         <v>20</v>
@@ -2124,7 +2124,7 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C40" t="s">
         <v>21</v>
@@ -2138,7 +2138,7 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
@@ -2152,7 +2152,7 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C42" t="s">
         <v>23</v>
@@ -2166,7 +2166,7 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C43" t="s">
         <v>24</v>
@@ -2180,7 +2180,7 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C44" t="s">
         <v>25</v>
@@ -2194,7 +2194,7 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C45" t="s">
         <v>26</v>
@@ -2208,7 +2208,7 @@
         <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C46" t="s">
         <v>27</v>
@@ -2222,10 +2222,10 @@
         <v>39</v>
       </c>
       <c r="C47" t="s">
+        <v>116</v>
+      </c>
+      <c r="D47" t="s">
         <v>117</v>
-      </c>
-      <c r="D47" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2236,7 +2236,7 @@
         <v>28</v>
       </c>
       <c r="D48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updating vignette for selectivity
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -186,9 +186,6 @@
     <t>Species number</t>
   </si>
   <si>
-    <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2. Not used otherwise</t>
-  </si>
-  <si>
     <t>Units used for survey: 1 = kg; 2 = numbers</t>
   </si>
   <si>
@@ -357,9 +354,6 @@
     <t>Variance of q prior: dnorm (log_q, log_q_prior, q_sd_prior)</t>
   </si>
   <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity, or descending logistic. 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic only. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
-  </si>
-  <si>
     <t>Wether a time-varying q should be estimated. 0 = no, 1 = penalized deviate, 2 = random effect, 3 = time blocks with no penalty; 4 = random walk from mean following Dorn 2018 (dnorm(q_y - q_y-1, 0, sigma). If Estimate_q = 5, this determines the environmental index to be used in the equation log(q_y) = q_mu + beta * index_y</t>
   </si>
   <si>
@@ -502,6 +496,12 @@
   </si>
   <si>
     <t>Selectivity to use for the species: 0 = empirical selectivity provided in srv_emp_sel; 1 = logistic selectivity; 2 = non-parametric selecitivty sensu Ianelli et al 2018; 3 = double logistic; 4 = descending logistic; 5 = non-parametric selectivity sensu Taylor et al 2014 (Hake)</t>
+  </si>
+  <si>
+    <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2 &amp; 5. Not used otherwise</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic only. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
   </si>
 </sst>
 </file>
@@ -1343,7 +1343,7 @@
         <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>30</v>
@@ -1352,7 +1352,7 @@
         <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>30</v>
@@ -1363,22 +1363,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" t="s">
         <v>85</v>
       </c>
-      <c r="F2" t="s">
-        <v>86</v>
-      </c>
       <c r="G2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1386,22 +1386,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1409,22 +1409,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" t="s">
         <v>90</v>
-      </c>
-      <c r="G4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1432,16 +1432,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" t="s">
         <v>135</v>
       </c>
-      <c r="C5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" t="s">
-        <v>137</v>
-      </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F5" t="s">
         <v>48</v>
@@ -1455,22 +1455,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1478,22 +1478,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F7" t="s">
         <v>49</v>
       </c>
       <c r="G7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1501,22 +1501,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F8" t="s">
         <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>55</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1524,22 +1524,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G9" t="s">
-        <v>112</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1547,22 +1547,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1570,22 +1570,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C11" t="s">
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" t="s">
         <v>93</v>
-      </c>
-      <c r="G11" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1593,22 +1593,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F12" t="s">
+        <v>94</v>
+      </c>
+      <c r="G12" t="s">
         <v>95</v>
-      </c>
-      <c r="G12" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1616,22 +1616,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
+        <v>96</v>
+      </c>
+      <c r="G13" t="s">
         <v>97</v>
-      </c>
-      <c r="G13" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1639,22 +1639,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D14" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
         <v>61</v>
-      </c>
-      <c r="G14" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1662,22 +1662,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F15" t="s">
         <v>52</v>
       </c>
       <c r="G15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1685,22 +1685,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F16" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1708,22 +1708,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C17" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D17" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" t="s">
         <v>74</v>
-      </c>
-      <c r="G17" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1731,22 +1731,22 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C18" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D18" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F18" t="s">
         <v>53</v>
       </c>
       <c r="G18" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1754,22 +1754,22 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D19" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1777,22 +1777,22 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C20" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D20" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1800,22 +1800,22 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C21" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D21" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G21" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1823,19 +1823,19 @@
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1849,13 +1849,13 @@
         <v>32</v>
       </c>
       <c r="E23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1869,13 +1869,13 @@
         <v>31</v>
       </c>
       <c r="E24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1883,19 +1883,19 @@
         <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D25" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1903,19 +1903,19 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1926,16 +1926,16 @@
         <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" t="s">
         <v>103</v>
-      </c>
-      <c r="G27" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1949,13 +1949,13 @@
         <v>33</v>
       </c>
       <c r="E28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F28" t="s">
         <v>51</v>
       </c>
       <c r="G28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1969,13 +1969,13 @@
         <v>34</v>
       </c>
       <c r="E29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F29" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G29" t="s">
         <v>105</v>
-      </c>
-      <c r="G29" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1989,10 +1989,10 @@
         <v>36</v>
       </c>
       <c r="F30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -2028,7 +2028,7 @@
         <v>39</v>
       </c>
       <c r="F33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2042,7 +2042,7 @@
         <v>40</v>
       </c>
       <c r="F34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2050,16 +2050,16 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
       </c>
       <c r="D35" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2067,13 +2067,13 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D36" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2081,13 +2081,13 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C37" t="s">
         <v>18</v>
       </c>
       <c r="D37" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F37" s="4"/>
     </row>
@@ -2096,13 +2096,13 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2110,7 +2110,7 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C39" t="s">
         <v>20</v>
@@ -2124,7 +2124,7 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
         <v>21</v>
@@ -2138,7 +2138,7 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
@@ -2152,7 +2152,7 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C42" t="s">
         <v>23</v>
@@ -2166,7 +2166,7 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C43" t="s">
         <v>24</v>
@@ -2180,7 +2180,7 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C44" t="s">
         <v>25</v>
@@ -2194,7 +2194,7 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C45" t="s">
         <v>26</v>
@@ -2208,7 +2208,7 @@
         <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C46" t="s">
         <v>27</v>
@@ -2222,10 +2222,10 @@
         <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D47" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2236,7 +2236,7 @@
         <v>28</v>
       </c>
       <c r="D48" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated multispecies modes and suitability estimation
Updated kinzey and punt 2009 multispecies modes and likelihoods
-multinomial diet prop fit
-lognromal ration fit
Updated lognormal and gamma suitability
Updated vignette
Still a bug or two need to address
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -15,6 +15,7 @@
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -483,9 +484,6 @@
     <t>Integer: switch to estimate or fix numbers-at-age: 0 = estimate dynamics, 1 = use input numbers-at-age in NbyageFixed, 2 = multiply input numbers-at-age (NbyageFixed) by a single scaling coefficient, 3 = multiply input numbers-at-age (NbyageFixed) by age specific scaling coefficient.</t>
   </si>
   <si>
-    <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: 1 = Exponential (Stewart et al 1983), 2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015), 3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979)</t>
-  </si>
-  <si>
     <t>Integer: which environmental index in env_data to use to drive bioenergetics</t>
   </si>
   <si>
@@ -502,6 +500,9 @@
   </si>
   <si>
     <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic only. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: 1 = Exponential (Stewart et al 1983), 2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015), 3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979); 4 = 1 for direct input of consumption in Pyrs  where consumption at age = Wt * Pyrs (CA set to 1, fday set to 1, CB set to 0)</t>
   </si>
 </sst>
 </file>
@@ -1493,7 +1494,7 @@
         <v>49</v>
       </c>
       <c r="G7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1516,7 +1517,7 @@
         <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1539,7 +1540,7 @@
         <v>67</v>
       </c>
       <c r="G9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -2056,7 +2057,7 @@
         <v>17</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="F35" t="s">
         <v>75</v>
@@ -2073,7 +2074,7 @@
         <v>113</v>
       </c>
       <c r="D36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2087,7 +2088,7 @@
         <v>18</v>
       </c>
       <c r="D37" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F37" s="4"/>
     </row>
@@ -2102,7 +2103,7 @@
         <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
remove Mn_LatAge and UobsAge
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -15,12 +15,11 @@
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="157">
   <si>
     <t>nspp</t>
   </si>
@@ -67,9 +66,6 @@
     <t>M1_base</t>
   </si>
   <si>
-    <t>Mn_LatAge</t>
-  </si>
-  <si>
     <t>aLW</t>
   </si>
   <si>
@@ -139,9 +135,6 @@
     <t>Residual natural mortality for each species</t>
   </si>
   <si>
-    <t>Mean length-at-age for each species. Used when estimating time-invariant length-based gamma suitability (suitMode = 1) or time invariant length-based lognormal suitability (suitMode = 4)</t>
-  </si>
-  <si>
     <t>Parameters for weight-at-length power function for each species. . Used when estimating time-variant length-based gamma suitability (suitMode = 2) or time-variant length-based lognormal suitability (suitMode = 5)</t>
   </si>
   <si>
@@ -154,13 +147,7 @@
     <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
   </si>
   <si>
-    <t>UobsAge</t>
-  </si>
-  <si>
     <t>UobsWtAge</t>
-  </si>
-  <si>
-    <t>Stomach proportion by numbers for each predator, prey, predator age, prey age combination. Can also be year specific by including the column, "Year"</t>
   </si>
   <si>
     <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Can also be year specific by including the column, "Year"</t>
@@ -1326,7 +1313,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -1338,25 +1325,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1364,22 +1351,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1387,22 +1374,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" t="s">
         <v>84</v>
-      </c>
-      <c r="F3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1410,22 +1397,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1433,22 +1420,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1456,22 +1443,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1479,22 +1466,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" t="s">
         <v>133</v>
       </c>
-      <c r="C7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" t="s">
-        <v>137</v>
-      </c>
       <c r="E7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1502,22 +1489,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1525,22 +1512,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G9" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1548,22 +1535,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1571,22 +1558,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s">
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E11" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G11" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1594,22 +1581,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1617,22 +1604,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F13" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G13" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1640,22 +1627,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C14" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D14" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1663,22 +1650,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" t="s">
         <v>52</v>
-      </c>
-      <c r="G15" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1686,22 +1673,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E16" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F16" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G16" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1709,22 +1696,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D17" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1732,22 +1719,22 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C18" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D18" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F18" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G18" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1755,22 +1742,22 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C19" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D19" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E19" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G19" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1778,22 +1765,22 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D20" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E20" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G20" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1801,22 +1788,22 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C21" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E21" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G21" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1824,19 +1811,19 @@
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D22" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E22" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F22" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G22" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1847,16 +1834,16 @@
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G23" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1867,16 +1854,16 @@
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E24" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G24" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1884,19 +1871,19 @@
         <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D25" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E25" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G25" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1904,19 +1891,19 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D26" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E26" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G26" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1927,16 +1914,16 @@
         <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E27" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G27" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1947,16 +1934,16 @@
         <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E28" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F28" t="s">
+        <v>47</v>
+      </c>
+      <c r="G28" t="s">
         <v>51</v>
-      </c>
-      <c r="G28" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1967,16 +1954,16 @@
         <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="G29" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1987,13 +1974,13 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F30" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="G30" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -2004,7 +1991,7 @@
         <v>13</v>
       </c>
       <c r="D31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -2015,7 +2002,7 @@
         <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2026,24 +2013,27 @@
         <v>15</v>
       </c>
       <c r="D33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F33" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>26</v>
       </c>
+      <c r="B34" t="s">
+        <v>130</v>
+      </c>
       <c r="C34" t="s">
         <v>16</v>
       </c>
       <c r="D34" t="s">
-        <v>40</v>
+        <v>156</v>
       </c>
       <c r="F34" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2051,16 +2041,16 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="D35" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F35" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2068,13 +2058,13 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s">
-        <v>113</v>
+        <v>17</v>
       </c>
       <c r="D36" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2082,13 +2072,13 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C37" t="s">
         <v>18</v>
       </c>
       <c r="D37" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F37" s="4"/>
     </row>
@@ -2097,13 +2087,13 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>156</v>
+        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2111,13 +2101,13 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C39" t="s">
         <v>20</v>
       </c>
       <c r="D39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2125,13 +2115,13 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C40" t="s">
         <v>21</v>
       </c>
       <c r="D40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2139,13 +2129,13 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2153,13 +2143,13 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C42" t="s">
         <v>23</v>
       </c>
       <c r="D42" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2167,13 +2157,13 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C43" t="s">
         <v>24</v>
       </c>
       <c r="D43" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2181,13 +2171,13 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C44" t="s">
         <v>25</v>
       </c>
       <c r="D44" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2195,27 +2185,24 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C45" t="s">
         <v>26</v>
       </c>
       <c r="D45" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>38</v>
       </c>
-      <c r="B46" t="s">
-        <v>134</v>
-      </c>
       <c r="C46" t="s">
-        <v>27</v>
+        <v>110</v>
       </c>
       <c r="D46" t="s">
-        <v>43</v>
+        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2223,10 +2210,10 @@
         <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>114</v>
+        <v>27</v>
       </c>
       <c r="D47" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2234,32 +2221,10 @@
         <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D48" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>41</v>
-      </c>
-      <c r="C49" t="s">
-        <v>44</v>
-      </c>
-      <c r="D49" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>42</v>
-      </c>
-      <c r="C50" t="s">
-        <v>45</v>
-      </c>
-      <c r="D50" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update random selectivity deviate switches
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -342,9 +342,6 @@
     <t>Variance of q prior: dnorm (log_q, log_q_prior, q_sd_prior)</t>
   </si>
   <si>
-    <t>Wether a time-varying q should be estimated. 0 = no, 1 = penalized deviate, 2 = random effect, 3 = time blocks with no penalty; 4 = random walk from mean following Dorn 2018 (dnorm(q_y - q_y-1, 0, sigma). If Estimate_q = 5, this determines the environmental index to be used in the equation log(q_y) = q_mu + beta * index_y</t>
-  </si>
-  <si>
     <t>Estimate catchability? (0 = fixed at prior; - 1 = Estimate single parameter; - 2 = Estimate single parameter with prior; - 3 = Estimate analytical q  from Ludwig and Walters 1994;  - 4 = Estimate power equation; - 5 - Linear equation log(q_y) = q_mu + beta * index_y)</t>
   </si>
   <si>
@@ -480,10 +477,13 @@
     <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2 &amp; 5. Not used otherwise</t>
   </si>
   <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). 0 = no, 1 = penalized deviates given sel_sd_prior, 2 = random effect, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic only. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
-  </si>
-  <si>
     <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: 1 = Exponential (Stewart et al 1983), 2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015), 3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979); 4 = 1 for direct input of consumption in Pyrs  where consumption at age = Wt * Pyrs (CA set to 1, fday set to 1, CB set to 0)</t>
+  </si>
+  <si>
+    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). 0 = no, 1 = penalized deviates given sel_sd_prior, 3 = time blocks with no penality, 4 = random walk following Dorn, 5 = random walk on ascending portion of double logistic only. If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity. "random_sel" treats random deviates and random walk parameters as random effects.</t>
+  </si>
+  <si>
+    <t>Wether a time-varying q should be estimated. 0 = no, 1 = penalized deviate, 3 = time blocks with no penalty; 4 = random walk from mean following Dorn 2018 (dnorm(q_y - q_y-1, 0, sigma). If Estimate_q = 5, this determines the environmental index to be used in the equation log(q_y) = q_mu + beta * index_y. If "random_q" is selected in fit_mod, penalized deviates (1) and random walk parameters (4) will be treated as random effects.</t>
   </si>
 </sst>
 </file>
@@ -1325,7 +1325,7 @@
         <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>29</v>
@@ -1345,13 +1345,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E2" t="s">
         <v>80</v>
@@ -1368,13 +1368,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
         <v>80</v>
@@ -1391,13 +1391,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E4" t="s">
         <v>80</v>
@@ -1414,13 +1414,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C5" t="s">
         <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E5" t="s">
         <v>80</v>
@@ -1437,13 +1437,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C6" t="s">
         <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E6" t="s">
         <v>80</v>
@@ -1452,7 +1452,7 @@
         <v>68</v>
       </c>
       <c r="G6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1460,13 +1460,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s">
         <v>74</v>
       </c>
       <c r="D7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E7" t="s">
         <v>80</v>
@@ -1475,7 +1475,7 @@
         <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1483,13 +1483,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
         <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E8" t="s">
         <v>80</v>
@@ -1498,7 +1498,7 @@
         <v>46</v>
       </c>
       <c r="G8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1506,13 +1506,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E9" t="s">
         <v>80</v>
@@ -1529,13 +1529,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
         <v>76</v>
       </c>
       <c r="D10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E10" t="s">
         <v>80</v>
@@ -1552,13 +1552,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C11" t="s">
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E11" t="s">
         <v>80</v>
@@ -1575,13 +1575,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E12" t="s">
         <v>80</v>
@@ -1598,13 +1598,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C13" t="s">
         <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E13" t="s">
         <v>80</v>
@@ -1621,13 +1621,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E14" t="s">
         <v>80</v>
@@ -1644,13 +1644,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C15" t="s">
         <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E15" t="s">
         <v>80</v>
@@ -1667,22 +1667,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E16" t="s">
         <v>80</v>
       </c>
       <c r="F16" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" t="s">
         <v>120</v>
-      </c>
-      <c r="G16" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1690,13 +1690,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E17" t="s">
         <v>80</v>
@@ -1713,13 +1713,13 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" t="s">
         <v>126</v>
-      </c>
-      <c r="D18" t="s">
-        <v>127</v>
       </c>
       <c r="E18" t="s">
         <v>80</v>
@@ -1728,7 +1728,7 @@
         <v>49</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1736,13 +1736,13 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E19" t="s">
         <v>80</v>
@@ -1759,13 +1759,13 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E20" t="s">
         <v>80</v>
@@ -1794,7 +1794,7 @@
         <v>65</v>
       </c>
       <c r="G21" t="s">
-        <v>107</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1842,10 +1842,10 @@
         <v>16</v>
       </c>
       <c r="C24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" t="s">
         <v>114</v>
-      </c>
-      <c r="D24" t="s">
-        <v>115</v>
       </c>
       <c r="E24" t="s">
         <v>80</v>
@@ -1862,10 +1862,10 @@
         <v>17</v>
       </c>
       <c r="C25" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" t="s">
         <v>112</v>
-      </c>
-      <c r="D25" t="s">
-        <v>113</v>
       </c>
       <c r="E25" t="s">
         <v>80</v>
@@ -1885,7 +1885,7 @@
         <v>9</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E26" t="s">
         <v>80</v>
@@ -2001,13 +2001,13 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C33" t="s">
         <v>16</v>
       </c>
       <c r="D33" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F33" t="s">
         <v>55</v>
@@ -2018,13 +2018,13 @@
         <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F34" t="s">
         <v>62</v>
@@ -2035,13 +2035,13 @@
         <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
       </c>
       <c r="D35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F35" t="s">
         <v>71</v>
@@ -2052,13 +2052,13 @@
         <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C36" t="s">
         <v>18</v>
       </c>
       <c r="D36" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2066,7 +2066,7 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C37" t="s">
         <v>19</v>
@@ -2081,7 +2081,7 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C38" t="s">
         <v>20</v>
@@ -2095,7 +2095,7 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C39" t="s">
         <v>21</v>
@@ -2109,7 +2109,7 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
@@ -2123,7 +2123,7 @@
         <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C41" t="s">
         <v>23</v>
@@ -2137,7 +2137,7 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C42" t="s">
         <v>24</v>
@@ -2151,7 +2151,7 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C43" t="s">
         <v>25</v>
@@ -2165,7 +2165,7 @@
         <v>36</v>
       </c>
       <c r="B44" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C44" t="s">
         <v>26</v>
@@ -2179,10 +2179,10 @@
         <v>37</v>
       </c>
       <c r="C45" t="s">
+        <v>109</v>
+      </c>
+      <c r="D45" t="s">
         <v>110</v>
-      </c>
-      <c r="D45" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2193,7 +2193,7 @@
         <v>27</v>
       </c>
       <c r="D46" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix random walk estimation and init edit
Keeps mean parameter, but turns off first dev.
Finit now = 0 if initMode != 3
Selectivity normalization turned on for Age_max_selected
- if negative, normalizes by max
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11207"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96251511-3738-954F-96A4-1F55F65F221A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4630FE8B-3C65-534F-A794-743F0BED64D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35760" yWindow="2340" windowWidth="31540" windowHeight="18100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="155">
   <si>
     <t>nspp</t>
   </si>
@@ -479,6 +479,12 @@
   </si>
   <si>
     <t>catch_data</t>
+  </si>
+  <si>
+    <t>Age_max_selected</t>
+  </si>
+  <si>
+    <t>Age at which selectivity = 1. If NA, it will not normalize selectivity. If &lt; 0, will normalize selectivity by the max.</t>
   </si>
 </sst>
 </file>
@@ -1579,10 +1585,10 @@
         <v>76</v>
       </c>
       <c r="F12" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1601,11 +1607,11 @@
       <c r="E13" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>54</v>
+      <c r="F13" t="s">
+        <v>147</v>
       </c>
       <c r="G13" t="s">
-        <v>55</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1624,11 +1630,11 @@
       <c r="E14" t="s">
         <v>76</v>
       </c>
-      <c r="F14" t="s">
-        <v>46</v>
+      <c r="F14" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1648,10 +1654,10 @@
         <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="G15" t="s">
-        <v>112</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1671,10 +1677,10 @@
         <v>76</v>
       </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>111</v>
       </c>
       <c r="G16" t="s">
-        <v>66</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1694,10 +1700,10 @@
         <v>76</v>
       </c>
       <c r="F17" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="G17" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1716,11 +1722,11 @@
       <c r="E18" t="s">
         <v>76</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>96</v>
+      <c r="F18" t="s">
+        <v>47</v>
       </c>
       <c r="G18" t="s">
-        <v>51</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1739,11 +1745,11 @@
       <c r="E19" t="s">
         <v>76</v>
       </c>
-      <c r="F19" t="s">
-        <v>62</v>
+      <c r="F19" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="G19" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1763,10 +1769,10 @@
         <v>76</v>
       </c>
       <c r="F20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G20" t="s">
-        <v>146</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1783,10 +1789,10 @@
         <v>76</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="G21" t="s">
-        <v>63</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1802,11 +1808,11 @@
       <c r="E22" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>87</v>
+      <c r="F22" t="s">
+        <v>97</v>
       </c>
       <c r="G22" t="s">
-        <v>150</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1823,10 +1829,10 @@
         <v>76</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G23" t="s">
-        <v>56</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1843,10 +1849,10 @@
         <v>76</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G24" t="s">
-        <v>151</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1863,10 +1869,10 @@
         <v>76</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G25" t="s">
-        <v>57</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1883,10 +1889,10 @@
         <v>76</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G26" t="s">
-        <v>91</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1902,11 +1908,11 @@
       <c r="E27" t="s">
         <v>76</v>
       </c>
-      <c r="F27" t="s">
-        <v>45</v>
+      <c r="F27" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="G27" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1922,11 +1928,11 @@
       <c r="E28" t="s">
         <v>76</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>92</v>
+      <c r="F28" t="s">
+        <v>45</v>
       </c>
       <c r="G28" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1942,6 +1948,12 @@
       <c r="E29" t="s">
         <v>76</v>
       </c>
+      <c r="F29" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G29" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
@@ -1953,11 +1965,8 @@
       <c r="D30" t="s">
         <v>34</v>
       </c>
-      <c r="F30" t="s">
-        <v>75</v>
-      </c>
-      <c r="G30" t="s">
-        <v>94</v>
+      <c r="E30" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1969,6 +1978,12 @@
       </c>
       <c r="D31" t="s">
         <v>35</v>
+      </c>
+      <c r="F31" t="s">
+        <v>75</v>
+      </c>
+      <c r="G31" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Revert "Merge branch 'dev-name-change' into dev"
This reverts commit 39b5f582ab46ab35880bbe642ffd6531a808ee69, reversing
changes made to 250c2c32c353e55009225b26c5fa39514086b8fe.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11207"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grant.adams\GitHub\Rceattle\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0872DD-B699-47F9-A158-D628F2BC7191}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4630FE8B-3C65-534F-A794-743F0BED64D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="765" windowWidth="34560" windowHeight="21585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="155">
   <si>
     <t>nspp</t>
   </si>
@@ -142,6 +142,9 @@
     <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
   </si>
   <si>
+    <t>UobsWtAge</t>
+  </si>
+  <si>
     <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Can also be year specific by including the column, "Year"</t>
   </si>
   <si>
@@ -232,6 +235,9 @@
     <t>spawn_month</t>
   </si>
   <si>
+    <t>R_sexr</t>
+  </si>
+  <si>
     <t>minage</t>
   </si>
   <si>
@@ -358,9 +364,21 @@
     <t>Age transition matrix (e.g. growth trajectory) used to convert age to length for length comp data. Can have multiple matrices for a species specified by Age_transition_index.</t>
   </si>
   <si>
+    <t>est_sex_ratio</t>
+  </si>
+  <si>
+    <t>sex_ratio_sigma</t>
+  </si>
+  <si>
     <t>estDynamics</t>
   </si>
   <si>
+    <t>proj_F</t>
+  </si>
+  <si>
+    <t>Unused</t>
+  </si>
+  <si>
     <t>Control</t>
   </si>
   <si>
@@ -376,6 +394,9 @@
     <t>Numeric: spawning month of the population to adjust the numbers at spawning</t>
   </si>
   <si>
+    <t>Numeric: percent of recruitment that is female (ignored if nsex = 1)</t>
+  </si>
+  <si>
     <t>Integer: end year of the hindcast</t>
   </si>
   <si>
@@ -409,6 +430,12 @@
     <t>Numeric: other food in the ecosystem for each species (kg)</t>
   </si>
   <si>
+    <t>Integer: is sex ration F/(M+F) to be included in the likelihood (assumed normal); 0 = no, 1 = use annual average across ages (uses 2nd age in propF data), 2 = age, and year specific (TBD)</t>
+  </si>
+  <si>
+    <t>Numeric: initial value or fixed value for sd of normal likelihood for sex ration. Not yet able to estimate.</t>
+  </si>
+  <si>
     <t>Integer: switch to estimate or fix numbers-at-age: 0 = estimate dynamics, 1 = use input numbers-at-age in NbyageFixed, 2 = multiply input numbers-at-age (NbyageFixed) by a single scaling coefficient, 3 = multiply input numbers-at-age (NbyageFixed) by age specific scaling coefficient.</t>
   </si>
   <si>
@@ -458,9 +485,6 @@
   </si>
   <si>
     <t>Age at which selectivity = 1. If NA, it will not normalize selectivity. If &lt; 0, will normalize selectivity by the max.</t>
-  </si>
-  <si>
-    <t>stom_prop_data</t>
   </si>
 </sst>
 </file>
@@ -1281,17 +1305,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G43"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="119.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="119.5" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1299,7 +1323,7 @@
         <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>27</v>
@@ -1308,824 +1332,880 @@
         <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" t="s">
+        <v>129</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" t="s">
+        <v>153</v>
+      </c>
+      <c r="G12" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" t="s">
+        <v>147</v>
+      </c>
+      <c r="G13" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" t="s">
+        <v>133</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>134</v>
+      </c>
+      <c r="E15" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>135</v>
+      </c>
+      <c r="E16" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" t="s">
+        <v>111</v>
+      </c>
+      <c r="G16" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18" t="s">
+        <v>118</v>
+      </c>
+      <c r="E18" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" t="s">
+        <v>47</v>
+      </c>
+      <c r="G18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" t="s">
+        <v>136</v>
+      </c>
+      <c r="E19" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" t="s">
+        <v>137</v>
+      </c>
+      <c r="E20" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" t="s">
+        <v>62</v>
+      </c>
+      <c r="G20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>13</v>
+      </c>
+      <c r="C21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>14</v>
+      </c>
+      <c r="C22" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" t="s">
+        <v>76</v>
+      </c>
+      <c r="F22" t="s">
+        <v>97</v>
+      </c>
+      <c r="G22" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
+        <v>152</v>
+      </c>
+      <c r="D23" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" t="s">
+        <v>106</v>
+      </c>
+      <c r="E24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G24" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>103</v>
+      </c>
+      <c r="D25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G25" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>18</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
         <v>113</v>
       </c>
-      <c r="C7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" t="s">
-        <v>117</v>
-      </c>
-      <c r="E7" t="s">
-        <v>74</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="E26" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>19</v>
+      </c>
+      <c r="C27" t="s">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
-        <v>113</v>
-      </c>
-      <c r="C8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" t="s">
-        <v>43</v>
-      </c>
-      <c r="G8" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="D27" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>20</v>
+      </c>
+      <c r="C28" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="D28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E28" t="s">
+        <v>76</v>
+      </c>
+      <c r="F28" t="s">
+        <v>45</v>
+      </c>
+      <c r="G28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>21</v>
+      </c>
+      <c r="C29" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G29" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>22</v>
+      </c>
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>23</v>
+      </c>
+      <c r="C31" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" t="s">
+        <v>35</v>
+      </c>
+      <c r="F31" t="s">
+        <v>75</v>
+      </c>
+      <c r="G31" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>24</v>
+      </c>
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>25</v>
+      </c>
+      <c r="B33" t="s">
+        <v>120</v>
+      </c>
+      <c r="C33" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" t="s">
+        <v>144</v>
+      </c>
+      <c r="F33" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>26</v>
+      </c>
+      <c r="B34" t="s">
+        <v>120</v>
+      </c>
+      <c r="C34" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" t="s">
+        <v>139</v>
+      </c>
+      <c r="F34" t="s">
         <v>58</v>
       </c>
-      <c r="G9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E10" t="s">
-        <v>74</v>
-      </c>
-      <c r="F10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" t="s">
-        <v>124</v>
-      </c>
-      <c r="E11" t="s">
-        <v>74</v>
-      </c>
-      <c r="F11" t="s">
-        <v>82</v>
-      </c>
-      <c r="G11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C12" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" t="s">
-        <v>125</v>
-      </c>
-      <c r="E12" t="s">
-        <v>74</v>
-      </c>
-      <c r="F12" t="s">
-        <v>144</v>
-      </c>
-      <c r="G12" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>113</v>
-      </c>
-      <c r="C13" t="s">
-        <v>108</v>
-      </c>
-      <c r="D13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" t="s">
-        <v>138</v>
-      </c>
-      <c r="G13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>113</v>
-      </c>
-      <c r="C14" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E14" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15">
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>27</v>
+      </c>
+      <c r="B35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C35" t="s">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
-        <v>113</v>
-      </c>
-      <c r="C15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" t="s">
-        <v>128</v>
-      </c>
-      <c r="E15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="D35" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>28</v>
+      </c>
+      <c r="B36" t="s">
+        <v>120</v>
+      </c>
+      <c r="C36" t="s">
         <v>16</v>
       </c>
-      <c r="B16" t="s">
-        <v>113</v>
-      </c>
-      <c r="C16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" t="s">
-        <v>129</v>
-      </c>
-      <c r="E16" t="s">
-        <v>74</v>
-      </c>
-      <c r="F16" t="s">
-        <v>109</v>
-      </c>
-      <c r="G16" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>13</v>
-      </c>
-      <c r="C17" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" t="s">
-        <v>93</v>
-      </c>
-      <c r="E17" t="s">
-        <v>74</v>
-      </c>
-      <c r="F17" t="s">
-        <v>64</v>
-      </c>
-      <c r="G17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>14</v>
-      </c>
-      <c r="C18" t="s">
-        <v>140</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="D36" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37">
         <v>29</v>
       </c>
-      <c r="E18" t="s">
-        <v>74</v>
-      </c>
-      <c r="F18" t="s">
-        <v>46</v>
-      </c>
-      <c r="G18" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>15</v>
-      </c>
-      <c r="C19" t="s">
-        <v>143</v>
-      </c>
-      <c r="D19" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" t="s">
-        <v>74</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="G19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>16</v>
-      </c>
-      <c r="C20" t="s">
-        <v>103</v>
-      </c>
-      <c r="D20" t="s">
-        <v>104</v>
-      </c>
-      <c r="E20" t="s">
-        <v>74</v>
-      </c>
-      <c r="F20" t="s">
-        <v>61</v>
-      </c>
-      <c r="G20" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21">
+      <c r="B37" t="s">
+        <v>120</v>
+      </c>
+      <c r="C37" t="s">
         <v>17</v>
       </c>
-      <c r="C21" t="s">
-        <v>101</v>
-      </c>
-      <c r="D21" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" t="s">
-        <v>74</v>
-      </c>
-      <c r="F21" t="s">
-        <v>60</v>
-      </c>
-      <c r="G21" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22">
+      <c r="D37" t="s">
+        <v>37</v>
+      </c>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>30</v>
+      </c>
+      <c r="B38" t="s">
+        <v>120</v>
+      </c>
+      <c r="C38" t="s">
         <v>18</v>
       </c>
-      <c r="C22" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" t="s">
-        <v>111</v>
-      </c>
-      <c r="E22" t="s">
-        <v>74</v>
-      </c>
-      <c r="F22" t="s">
-        <v>95</v>
-      </c>
-      <c r="G22" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23">
+      <c r="D38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>31</v>
+      </c>
+      <c r="B39" t="s">
+        <v>120</v>
+      </c>
+      <c r="C39" t="s">
         <v>19</v>
-      </c>
-      <c r="C23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" t="s">
-        <v>74</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G23" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>20</v>
-      </c>
-      <c r="C24" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" t="s">
-        <v>74</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>21</v>
-      </c>
-      <c r="C25" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" t="s">
-        <v>74</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G25" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>22</v>
-      </c>
-      <c r="C26" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" t="s">
-        <v>34</v>
-      </c>
-      <c r="E26" t="s">
-        <v>74</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G26" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>23</v>
-      </c>
-      <c r="C27" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" t="s">
-        <v>35</v>
-      </c>
-      <c r="E27" t="s">
-        <v>74</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G27" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>24</v>
-      </c>
-      <c r="C28" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" t="s">
-        <v>36</v>
-      </c>
-      <c r="E28" t="s">
-        <v>74</v>
-      </c>
-      <c r="F28" t="s">
-        <v>44</v>
-      </c>
-      <c r="G28" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>25</v>
-      </c>
-      <c r="B29" t="s">
-        <v>114</v>
-      </c>
-      <c r="C29" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" t="s">
-        <v>135</v>
-      </c>
-      <c r="E29" t="s">
-        <v>74</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>26</v>
-      </c>
-      <c r="B30" t="s">
-        <v>114</v>
-      </c>
-      <c r="C30" t="s">
-        <v>98</v>
-      </c>
-      <c r="D30" t="s">
-        <v>130</v>
-      </c>
-      <c r="E30" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>27</v>
-      </c>
-      <c r="B31" t="s">
-        <v>114</v>
-      </c>
-      <c r="C31" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" t="s">
-        <v>131</v>
-      </c>
-      <c r="F31" t="s">
-        <v>73</v>
-      </c>
-      <c r="G31" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>28</v>
-      </c>
-      <c r="B32" t="s">
-        <v>114</v>
-      </c>
-      <c r="C32" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>29</v>
-      </c>
-      <c r="B33" t="s">
-        <v>114</v>
-      </c>
-      <c r="C33" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" t="s">
-        <v>37</v>
-      </c>
-      <c r="F33" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>30</v>
-      </c>
-      <c r="B34" t="s">
-        <v>114</v>
-      </c>
-      <c r="C34" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" t="s">
-        <v>38</v>
-      </c>
-      <c r="F34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>31</v>
-      </c>
-      <c r="B35" t="s">
-        <v>114</v>
-      </c>
-      <c r="C35" t="s">
-        <v>19</v>
-      </c>
-      <c r="D35" t="s">
-        <v>39</v>
-      </c>
-      <c r="F35" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>32</v>
-      </c>
-      <c r="B36" t="s">
-        <v>114</v>
-      </c>
-      <c r="C36" t="s">
-        <v>20</v>
-      </c>
-      <c r="D36" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>33</v>
-      </c>
-      <c r="B37" t="s">
-        <v>114</v>
-      </c>
-      <c r="C37" t="s">
-        <v>21</v>
-      </c>
-      <c r="D37" t="s">
-        <v>39</v>
-      </c>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>34</v>
-      </c>
-      <c r="B38" t="s">
-        <v>114</v>
-      </c>
-      <c r="C38" t="s">
-        <v>22</v>
-      </c>
-      <c r="D38" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>35</v>
-      </c>
-      <c r="B39" t="s">
-        <v>114</v>
-      </c>
-      <c r="C39" t="s">
-        <v>23</v>
       </c>
       <c r="D39" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D40" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
+        <v>33</v>
+      </c>
+      <c r="B41" t="s">
+        <v>120</v>
+      </c>
+      <c r="C41" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>34</v>
+      </c>
+      <c r="B42" t="s">
+        <v>120</v>
+      </c>
+      <c r="C42" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>35</v>
+      </c>
+      <c r="B43" t="s">
+        <v>120</v>
+      </c>
+      <c r="C43" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>36</v>
+      </c>
+      <c r="B44" t="s">
+        <v>120</v>
+      </c>
+      <c r="C44" t="s">
+        <v>24</v>
+      </c>
+      <c r="D44" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45">
         <v>37</v>
       </c>
-      <c r="C41" t="s">
-        <v>99</v>
-      </c>
-      <c r="D41" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42">
+      <c r="C45" t="s">
+        <v>101</v>
+      </c>
+      <c r="D45" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46">
         <v>38</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C46" t="s">
         <v>25</v>
       </c>
-      <c r="D42" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43">
+      <c r="D46" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47">
         <v>39</v>
       </c>
-      <c r="C43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C47" t="s">
         <v>40</v>
+      </c>
+      <c r="D47" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upper age_max_selected for normalizing across range of ages
Switch checks as well
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grant.adams\GitHub\Rceattle\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF88D93E-E48A-4C47-950E-A281CB2CA96D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BD06EC-C598-4F3D-9E6F-C40129725B64}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="765" windowWidth="34560" windowHeight="21585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="143">
   <si>
     <t>nspp</t>
   </si>
@@ -492,6 +492,12 @@
   </si>
   <si>
     <t>Sheet name</t>
+  </si>
+  <si>
+    <t>Age_max_selected_upper</t>
+  </si>
+  <si>
+    <t>Upper age for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Age_max_selected` and `Age_max_selected_upper`</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1336,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="6" bestFit="1" customWidth="1"/>
@@ -1655,39 +1661,40 @@
       <c r="C28" s="4" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B29" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C30" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B30" s="7" t="s">
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C31" s="4" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1695,10 +1702,10 @@
         <v>56</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="C32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1706,234 +1713,234 @@
         <v>56</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="6" t="s">
+    <row r="35" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C35" s="4" t="s">
         <v>122</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C35" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C37" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B37" s="6" t="s">
+    <row r="38" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C38" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="2"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="6" t="s">
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B39" s="8" t="s">
+    <row r="40" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C40" s="4" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B40" s="8" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C41" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B41" s="8" t="s">
+    <row r="42" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C42" s="4" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B42" s="8" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C43" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B43" s="8" t="s">
+    <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B44" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C44" s="4" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C44" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>97</v>
+        <v>56</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>66</v>
       </c>
       <c r="C45" t="s">
-        <v>133</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C46" t="s">
-        <v>22</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C48" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C49" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+    <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C50" s="4" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C51" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
+    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C52" s="4" t="s">
         <v>135</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C52" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C53" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C54" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C55" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A56" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C57" t="s">
-        <v>92</v>
+        <v>10</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1941,10 +1948,10 @@
         <v>82</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="C58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1952,10 +1959,10 @@
         <v>82</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1963,10 +1970,10 @@
         <v>82</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C60" t="s">
-        <v>27</v>
+        <v>94</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1974,10 +1981,10 @@
         <v>82</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C61" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1985,10 +1992,10 @@
         <v>82</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C62" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1996,7 +2003,7 @@
         <v>82</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C63" t="s">
         <v>29</v>
@@ -2007,7 +2014,7 @@
         <v>82</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C64" t="s">
         <v>29</v>
@@ -2018,7 +2025,7 @@
         <v>82</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C65" t="s">
         <v>29</v>
@@ -2029,7 +2036,7 @@
         <v>82</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C66" t="s">
         <v>29</v>
@@ -2040,7 +2047,7 @@
         <v>82</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C67" t="s">
         <v>29</v>
@@ -2048,48 +2055,59 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>72</v>
+        <v>82</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="C68" t="s">
-        <v>137</v>
+        <v>29</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="C69" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C70" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C71" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A73" s="6" t="s">
+    <row r="74" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B73" s="9" t="s">
+      <c r="B74" s="9" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding weighted-mean diet data and documentation
Added weighted mean diet proportion of prey-spp in predator-spp (sum across prey ages and take weighted mean across predator ages)

Added documentation to meta_data about diet data options

Diet_data can now be predicted but not included in likelihood
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grant.adams\GitHub\Rceattle\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BD06EC-C598-4F3D-9E6F-C40129725B64}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8189E839-E1F0-4A38-84B5-E0BF69DEF48F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="765" windowWidth="34560" windowHeight="21585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="145">
   <si>
     <t>nspp</t>
   </si>
@@ -110,9 +110,6 @@
   </si>
   <si>
     <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
-  </si>
-  <si>
-    <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Can also be year specific by including the column, "Year"</t>
   </si>
   <si>
     <t>Species</t>
@@ -461,9 +458,6 @@
 After running model, these will update to McAllister &amp; Ianelli 1997 weights using the harmonic mean.</t>
   </si>
   <si>
-    <t>Survey index or fishery indices in weight (kg) or numbers</t>
-  </si>
-  <si>
     <t>Age transition matrix (e.g. growth trajectory) used to convert age to length for length comp data. 
 Can have multiple matrices for a species specified by Age_transition_index.</t>
   </si>
@@ -498,6 +492,24 @@
   </si>
   <si>
     <t>Upper age for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Age_max_selected` and `Age_max_selected_upper`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Survey index or fishery indices in weight (kg) or numbers. </t>
+  </si>
+  <si>
+    <t>NOTE: For catch, index, and comp data, if "Year" is negative, it will predict for that year, but not include the data in the likelihood.</t>
+  </si>
+  <si>
+    <t>NOTE: For emp_sel, weight, and ration_data, if "Year" == 0, those data will be used for all years</t>
+  </si>
+  <si>
+    <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Multiple diet-data formats can be included:
+1) If Pred_age &gt;= 0 and Prey_age &gt;= 0, data is assumed to be  diet proportion of prey-at-age/sex in predator-at-age/sex. 
+2) If Pred_age &gt;= 0 and Prey_age &lt; 0, data is assumed to be mean diet proportion of prey-spp in predator-at-age/sex (sum across prey ages and sexes)
+3) If Pred_age &lt; 0 and Prey_age &lt; 0, data is assumed to be  mean diet proportion of prey-spp in predator-spp (sum across prey ages/sexes and take mean across predator ages/sexes)
+4) If Pred_age &lt; -500 and Prey_age &lt; 0, data is assumed to be weighted mean diet proportion of prey-spp in predator-spp (sum across prey ages/sexes and take weighted mean across predator ages/sexes). Weights are estimated predators-at-age.
+If "Year = 0", the the diet will be assumed to be the average between "suit_styr" and "suit_endyr". 
+Only diet-data type 1 can be used for MSVPA based suitability</t>
   </si>
 </sst>
 </file>
@@ -1336,7 +1348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="6" bestFit="1" customWidth="1"/>
@@ -1348,10 +1360,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
@@ -1362,507 +1374,507 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E23" s="2"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E25" s="2"/>
     </row>
     <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" t="s">
         <v>61</v>
-      </c>
-      <c r="C27" t="s">
-        <v>62</v>
       </c>
       <c r="E27" s="2"/>
     </row>
     <row r="28" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E28" s="2"/>
     </row>
     <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E30" s="2"/>
     </row>
     <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" t="s">
         <v>46</v>
-      </c>
-      <c r="C34" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E38" s="2"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C39" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B41" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C41" t="s">
         <v>127</v>
-      </c>
-      <c r="C41" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C43" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B45" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" t="s">
         <v>66</v>
-      </c>
-      <c r="C45" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C46" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
@@ -1870,18 +1882,18 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" t="s">
         <v>75</v>
-      </c>
-      <c r="C48" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C49" t="s">
         <v>73</v>
-      </c>
-      <c r="C49" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1889,7 +1901,7 @@
         <v>7</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1902,15 +1914,15 @@
     </row>
     <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C53" t="s">
         <v>24</v>
@@ -1918,7 +1930,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C54" t="s">
         <v>25</v>
@@ -1934,51 +1946,51 @@
     </row>
     <row r="57" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C60" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>13</v>
@@ -1989,7 +2001,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>14</v>
@@ -2000,7 +2012,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>15</v>
@@ -2011,7 +2023,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>16</v>
@@ -2022,7 +2034,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>17</v>
@@ -2033,7 +2045,7 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>18</v>
@@ -2044,7 +2056,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>19</v>
@@ -2055,7 +2067,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>20</v>
@@ -2066,49 +2078,59 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C69" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C70" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="210" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C71" t="s">
-        <v>30</v>
+        <v>102</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="6" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CAAL updates - compiles and tests w/o CAAL data work
Refactor: Rename Pyrs to "ration_data", old name will still be read in, but name will be updated

Feature: Added internal growth calculation, see \code{build_growth} within \code{fit_mod} wrapper and growth.hpp. Added `beta_wt_len` and `alpha_wt_len` to "control" sheet of data. Added CAAL_loglike and CAAL_weights to fleet control. Added CAAL_data to data.

Feature: Added size based selectivity.

Feature: Added month to "fleet_control"

Refactor: Change Nselages to N_sel_bins

Refactor: renamed N_sel_bins = Nselages, Sel_norm_bin1 = Age_max_selected, and Sel_norm_bin2 = Age_max_selected_upper
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grant.adams\GitHub\Rceattle\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8189E839-E1F0-4A38-84B5-E0BF69DEF48F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6940EDAC-9B17-BB4F-88DF-FDDECB12F63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="765" windowWidth="34560" windowHeight="21585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="151">
   <si>
     <t>nspp</t>
   </si>
@@ -118,9 +118,6 @@
     <t>Selectivity</t>
   </si>
   <si>
-    <t>Nselages</t>
-  </si>
-  <si>
     <t>Weight_index</t>
   </si>
   <si>
@@ -205,9 +202,6 @@
     <t>Age_first_selected</t>
   </si>
   <si>
-    <t>Age at which selectivity is non-zero</t>
-  </si>
-  <si>
     <t>Estimate_catch_sd</t>
   </si>
   <si>
@@ -304,9 +298,6 @@
     <t>Numeric: number of foraging days per year for each species</t>
   </si>
   <si>
-    <t>Number of ages to estimate non-parametric selectivity for Selectivity = 2 &amp; 5. Not used otherwise</t>
-  </si>
-  <si>
     <t>Comp_loglike</t>
   </si>
   <si>
@@ -316,9 +307,6 @@
     <t>catch_data</t>
   </si>
   <si>
-    <t>Age_max_selected</t>
-  </si>
-  <si>
     <t>weight</t>
   </si>
   <si>
@@ -350,9 +338,6 @@
   </si>
   <si>
     <t>Index of survey/fishery (does not restart for each species)</t>
-  </si>
-  <si>
-    <t>Index to match selectivities (otherwise, same as fleet_code)</t>
   </si>
   <si>
     <t>Integer: switch to estimate or fix numbers-at-age: 
@@ -388,11 +373,6 @@
 If selectivity is set to type = 2 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
   </si>
   <si>
-    <t>Age at which selectivity = 1. 
-If NA, it will not normalize selectivity. 
-If &lt; 0, will normalize selectivity by the max.</t>
-  </si>
-  <si>
     <t>Composition data distribution:
 -1 = AFSC multinomial
 0 = full multinomial
@@ -466,13 +446,6 @@
 Can have multiple weight-at-age data-sets for each species.</t>
   </si>
   <si>
-    <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: 
-1 = Exponential (Stewart et al 1983)
-2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015)
-3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979)
-4 = for direct input of consumption in Pyrs  where consumption at age = Wt * Pyrs (CA set to 1, fday set to 1, CB set to 0)</t>
-  </si>
-  <si>
     <t>Environmental indices such as bottom temperature data to incorporate into ration equation specificed by Ceq and Cindex. Also used to drive catchability if Estimate_q = 5 or 6. Will use the mean for missing years. Temperature should be in celcius.</t>
   </si>
   <si>
@@ -486,12 +459,6 @@
   </si>
   <si>
     <t>Sheet name</t>
-  </si>
-  <si>
-    <t>Age_max_selected_upper</t>
-  </si>
-  <si>
-    <t>Upper age for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Age_max_selected` and `Age_max_selected_upper`</t>
   </si>
   <si>
     <t xml:space="preserve">Survey index or fishery indices in weight (kg) or numbers. </t>
@@ -510,6 +477,57 @@
 4) If Pred_age &lt; -500 and Prey_age &lt; 0, data is assumed to be weighted mean diet proportion of prey-spp in predator-spp (sum across prey ages/sexes and take weighted mean across predator ages/sexes). Weights are estimated predators-at-age.
 If "Year = 0", the the diet will be assumed to be the average between "suit_styr" and "suit_endyr". 
 Only diet-data type 1 can be used for MSVPA based suitability</t>
+  </si>
+  <si>
+    <t>alpha_wt_len</t>
+  </si>
+  <si>
+    <t>beta_wt_len</t>
+  </si>
+  <si>
+    <t>Alpha parameter from Weight = alpha * Length ^ beta</t>
+  </si>
+  <si>
+    <t>Beta parameter from Weight = alpha * Length ^ beta</t>
+  </si>
+  <si>
+    <t>Index to mirror selectivities (otherwise, same as fleet_code)</t>
+  </si>
+  <si>
+    <t>N_sel_bins</t>
+  </si>
+  <si>
+    <t>Number of age or length bins to estimate non-parametric selectivity for Selectivity = 2 &amp; 5. Not used otherwise</t>
+  </si>
+  <si>
+    <t>Sel_norm_bin1</t>
+  </si>
+  <si>
+    <t>Sel_norm_bin2</t>
+  </si>
+  <si>
+    <t>Upper age/length bin for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Age_max_selected` and `Age_max_selected_upper`</t>
+  </si>
+  <si>
+    <t>Age/length bin at which selectivity = 1. 
+If NA, it will not normalize selectivity. 
+If &lt; 0, will normalize selectivity by the max.</t>
+  </si>
+  <si>
+    <t>Age at which selectivity becomes non-zero</t>
+  </si>
+  <si>
+    <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: 
+1 = Exponential (Stewart et al 1983)
+2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015)
+3 = temperature dependence for cool and cold-water species (Thornton and Lessem 1979)
+4 = for direct input of consumption in Pyrs  where consumption at age = Numbers * Pyrs (CA set to 1, fday set to 1, CB set to 0)</t>
+  </si>
+  <si>
+    <t>caal_data</t>
+  </si>
+  <si>
+    <t>Survey/fishery CAAL data. Note if sex is 3, put female CAAL data then male CAAL data (similar to SS).</t>
   </si>
 </sst>
 </file>
@@ -1348,22 +1366,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F80"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F83"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="119.42578125" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.83203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="119.5" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
@@ -1372,765 +1390,795 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="6" t="s">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C26" t="s">
+        <v>142</v>
+      </c>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" ht="112" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" t="s">
+        <v>147</v>
+      </c>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="64" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="112" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C43" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C45" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C47" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C48" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C50" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C51" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C52" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="A55" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C56" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C57" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C61" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C62" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B16" s="6" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" t="s">
-        <v>109</v>
-      </c>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" t="s">
-        <v>94</v>
-      </c>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="1:5" ht="120" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C32" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C34" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C36" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="E38" s="2"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C39" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="C41" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C46" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C47" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C48" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C51" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A52" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C53" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C54" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C55" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A57" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C58" t="s">
+      <c r="B63" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C63" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C59" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C60" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B61" s="6" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B64" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C64" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B62" s="6" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B65" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C65" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B63" s="6" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B66" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="C63" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C64" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C65" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="C66" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C67" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C68" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
-        <v>71</v>
+        <v>79</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="C69" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C70" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C71" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C72" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C73" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C74" s="4" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C70" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A71" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A74" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B74" s="9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" ht="64" x14ac:dyDescent="0.2">
       <c r="A77" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="6" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="6" t="s">
-        <v>143</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83" s="6" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made sure size-selex works and added
refactor: changed Age_first_selected to Bin_first_selected
refactor: sel to sel_at_age
fix: small bugs
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6940EDAC-9B17-BB4F-88DF-FDDECB12F63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD74161-B810-414B-A58B-4F9D3E63D020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="155">
   <si>
     <t>nspp</t>
   </si>
@@ -197,9 +197,6 @@
   </si>
   <si>
     <t>Fleet_type</t>
-  </si>
-  <si>
-    <t>Age_first_selected</t>
   </si>
   <si>
     <t>Estimate_catch_sd</t>
@@ -350,27 +347,6 @@
     <t>0 = Do not estimate (fixes all parameters for this fleet to initial values)
 1 = Fishery
 2 = Survey</t>
-  </si>
-  <si>
-    <t>0 = empirical selectivity provided in srv_emp_sel
-1 = logistic selectivity
-2 = non-parametric selecitivty sensu Ianelli et al 2018
-3 = double logistic
-4 = descending logistic
-5 = non-parametric selectivity sensu Taylor et al 2014 (Hake)</t>
-  </si>
-  <si>
-    <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). 
-0 = no
-1 = penalized deviates given sel_sd_prior (or random effects if "random_sel" is selected in "fit_mod"), 
-3 = time blocks with no penality 
-4 = random walk following Dorn
-5 = random walk on ascending portion of double logistic only. 
-If selectivity is set to type = 2 (non-parametric) this value will be the 1st penalty on selectivity.</t>
-  </si>
-  <si>
-    <t>The sd to use for the random walk of time varying selectivity if set to 1. 
-If selectivity is set to type = 2 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
   </si>
   <si>
     <t>Composition data distribution:
@@ -514,9 +490,6 @@
 If &lt; 0, will normalize selectivity by the max.</t>
   </si>
   <si>
-    <t>Age at which selectivity becomes non-zero</t>
-  </si>
-  <si>
     <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: 
 1 = Exponential (Stewart et al 1983)
 2 = Temperature-dependendence for warm-water species (Kitchell et al 1977; sensu Holsman et al 2015)
@@ -528,6 +501,48 @@
   </si>
   <si>
     <t>Survey/fishery CAAL data. Note if sex is 3, put female CAAL data then male CAAL data (similar to SS).</t>
+  </si>
+  <si>
+    <t>Bin_first_selected</t>
+  </si>
+  <si>
+    <t>Age/length bin at which selectivity becomes non-zero</t>
+  </si>
+  <si>
+    <t>0 = empirical selectivity provided in srv_emp_sel
+1 = Age-based logistic selectivity
+2 = Age-based non-parametric selecitivty sensu Ianelli et al 2018
+3 = Age-based double logistic
+4 = Age-based descending logistic
+5 = Age-based non-parametric selectivity sensu Taylor et al 2014 (Hake)
+6 = Length-based logistic selectivity
+7 = Length-based non-parametric selecitivty sensu Ianelli et al 2018
+8 = Length-based double logistic
+9 = Length-based descending logistic
+10 = Length-based non-parametric selectivity sensu Taylor et al 2014 (Hake)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). 
+0 = no
+1 = penalized deviates given sel_sd_prior (or random effects if "random_sel" is selected in "fit_mod"), 
+3 = time blocks with no penality 
+4 = random walk following Dorn
+5 = random walk on ascending portion of double logistic only. </t>
+  </si>
+  <si>
+    <t>Sel_curve_pen1</t>
+  </si>
+  <si>
+    <t>Sel_curve_pen2</t>
+  </si>
+  <si>
+    <t>The sd to use for the random walk of time varying selectivity if set to 1, 4, or 5.</t>
+  </si>
+  <si>
+    <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 1st penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
   </si>
 </sst>
 </file>
@@ -1366,7 +1381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="6" bestFit="1" customWidth="1"/>
@@ -1378,10 +1393,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
@@ -1392,190 +1407,190 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>49</v>
       </c>
       <c r="C7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="80" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C17" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C18" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1584,7 +1599,7 @@
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1606,7 +1621,7 @@
         <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E21" s="2"/>
     </row>
@@ -1618,7 +1633,7 @@
         <v>58</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1640,10 +1655,10 @@
         <v>43</v>
       </c>
       <c r="C24" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="176" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>54</v>
       </c>
@@ -1651,7 +1666,7 @@
         <v>31</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>108</v>
+        <v>148</v>
       </c>
       <c r="E25" s="2"/>
     </row>
@@ -1660,81 +1675,82 @@
         <v>54</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C26" t="s">
+        <v>138</v>
+      </c>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" t="s">
+        <v>153</v>
+      </c>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C28" t="s">
+        <v>154</v>
+      </c>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" t="s">
+        <v>147</v>
+      </c>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="1:5" ht="112" x14ac:dyDescent="0.2">
-      <c r="A27" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" t="s">
-        <v>147</v>
-      </c>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A30" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A31" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="64" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>111</v>
       </c>
       <c r="E32" s="2"/>
     </row>
@@ -1742,33 +1758,34 @@
       <c r="A33" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="64" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C35" t="s">
-        <v>114</v>
+      <c r="C35" s="4" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1776,88 +1793,88 @@
         <v>54</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C36" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="112" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>115</v>
+        <v>75</v>
+      </c>
+      <c r="C37" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="8" t="s">
-        <v>66</v>
+      <c r="B38" s="6" t="s">
+        <v>44</v>
       </c>
       <c r="C38" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="112" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A40" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E40" s="2"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="C41" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="96" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="8" t="s">
-        <v>119</v>
+      <c r="B42" s="6" t="s">
+        <v>41</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>123</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="E42" s="2"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="8" t="s">
-        <v>120</v>
+      <c r="B43" s="6" t="s">
+        <v>66</v>
       </c>
       <c r="C43" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -1865,10 +1882,10 @@
         <v>54</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>60</v>
+        <v>115</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1876,21 +1893,21 @@
         <v>54</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="C45" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1898,194 +1915,194 @@
         <v>54</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C47" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C48" t="s">
-        <v>132</v>
+        <v>54</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
-        <v>94</v>
+        <v>54</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="C49" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="C50" t="s">
-        <v>73</v>
+        <v>128</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
-        <v>149</v>
+        <v>93</v>
       </c>
       <c r="C51" t="s">
-        <v>150</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C52" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>126</v>
+        <v>144</v>
+      </c>
+      <c r="C53" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="C54" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
-        <v>96</v>
+        <v>8</v>
       </c>
       <c r="C56" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C57" t="s">
-        <v>25</v>
+        <v>94</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C58" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C59" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C60" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="80" x14ac:dyDescent="0.2">
-      <c r="A60" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B60" s="6" t="s">
+    <row r="62" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C60" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C61" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C62" t="s">
-        <v>90</v>
+      <c r="C62" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="C63" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>27</v>
+        <v>89</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C65" t="s">
-        <v>28</v>
+        <v>90</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C66" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C67" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C68" t="s">
         <v>29</v>
@@ -2093,10 +2110,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C69" t="s">
         <v>29</v>
@@ -2104,10 +2121,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C70" t="s">
         <v>29</v>
@@ -2115,10 +2132,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C71" t="s">
         <v>29</v>
@@ -2126,59 +2143,81 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
-        <v>69</v>
+        <v>78</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="C72" t="s">
-        <v>128</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
-        <v>99</v>
+        <v>78</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="C73" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C74" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C74" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" ht="64" x14ac:dyDescent="0.2">
-      <c r="A77" s="6" t="s">
+      <c r="C75" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+      <c r="A79" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B77" s="9" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="6" t="s">
-        <v>38</v>
+      <c r="B79" s="9" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" s="6" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="6" t="s">
-        <v>133</v>
+        <v>38</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" s="6" t="s">
-        <v>134</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A85" s="6" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tests, examples, and renames
rename "Catchability" to "Catchability"
rename: "Time_varying_sel_sd_prior" to "Time_varying_sel_sd_prior"
feature: added CAAL data simulation to sim_mod
feature: added CAAL data update run_mse
fix: added check of column names for sex_ratio and maturity to deal with contains("Age") for selecting the columns
Double checked tests and examples to make sure things are running
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD74161-B810-414B-A58B-4F9D3E63D020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0A6E23-7146-7249-BECD-2D0D2B1F9B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="159">
   <si>
     <t>nspp</t>
   </si>
@@ -121,9 +121,6 @@
     <t>Weight_index</t>
   </si>
   <si>
-    <t>Estimate_q</t>
-  </si>
-  <si>
     <t>Species number</t>
   </si>
   <si>
@@ -140,9 +137,6 @@
   </si>
   <si>
     <t>Time_varying_sel</t>
-  </si>
-  <si>
-    <t>Sel_sd_prior</t>
   </si>
   <si>
     <t>Time_varying_q</t>
@@ -536,13 +530,33 @@
     <t>Sel_curve_pen2</t>
   </si>
   <si>
-    <t>The sd to use for the random walk of time varying selectivity if set to 1, 4, or 5.</t>
-  </si>
-  <si>
     <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 1st penalty on selectivity.</t>
   </si>
   <si>
     <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
+  </si>
+  <si>
+    <t>The fixed or initial sd to use for time varying selectivity if set to 1, 4, or 5.</t>
+  </si>
+  <si>
+    <t>Time_varying_sel_sd_prior</t>
+  </si>
+  <si>
+    <t>Catchability</t>
+  </si>
+  <si>
+    <t>CAAL_loglike</t>
+  </si>
+  <si>
+    <t>CAAL_weights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composition weights for CAAL  likelihood. </t>
+  </si>
+  <si>
+    <t>Composition data distribution:
+0 = full multinomial
+1 = dirichlet-multinomial</t>
   </si>
 </sst>
 </file>
@@ -1381,7 +1395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="6" bestFit="1" customWidth="1"/>
@@ -1393,10 +1407,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
@@ -1407,323 +1421,323 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
         <v>77</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="80" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" t="s">
         <v>132</v>
-      </c>
-      <c r="C17" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" t="s">
         <v>133</v>
-      </c>
-      <c r="C18" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s">
         <v>55</v>
-      </c>
-      <c r="C20" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>56</v>
-      </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C24" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="176" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>31</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E25" s="2"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C26" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C27" t="s">
         <v>150</v>
-      </c>
-      <c r="C27" t="s">
-        <v>153</v>
       </c>
       <c r="E27" s="2"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C28" t="s">
         <v>151</v>
-      </c>
-      <c r="C28" t="s">
-        <v>154</v>
       </c>
       <c r="E28" s="2"/>
     </row>
     <row r="29" spans="1:5" ht="96" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E29" s="2"/>
     </row>
     <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>40</v>
+        <v>153</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>152</v>
@@ -1732,247 +1746,255 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C31" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E31" s="2"/>
     </row>
     <row r="32" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E32" s="2"/>
     </row>
     <row r="33" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="64" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E34" s="2"/>
+        <v>105</v>
+      </c>
     </row>
     <row r="35" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>37</v>
+        <v>52</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C36" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="112" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>111</v>
+      <c r="C39" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>65</v>
+        <v>52</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>73</v>
       </c>
       <c r="C40" t="s">
-        <v>35</v>
+        <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>42</v>
       </c>
       <c r="C41" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="112" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>41</v>
+        <v>154</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="E42" s="2"/>
+        <v>109</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>66</v>
+        <v>52</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="C43" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C46" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B48" s="8" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A44" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B44" s="8" t="s">
+      <c r="C48" t="s">
         <v>115</v>
       </c>
-      <c r="C44" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B45" s="8" t="s">
+    </row>
+    <row r="49" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="A49" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="C45" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C47" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A48" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C49" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
-        <v>92</v>
+        <v>52</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="C50" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
-        <v>93</v>
+        <v>52</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="C51" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s">
-        <v>72</v>
+        <v>126</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>145</v>
+        <v>22</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -1983,148 +2005,142 @@
         <v>70</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>122</v>
+        <v>142</v>
+      </c>
+      <c r="C55" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
-        <v>8</v>
+        <v>67</v>
       </c>
       <c r="C56" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
-        <v>94</v>
+        <v>7</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="C58" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C59" t="s">
-        <v>25</v>
+        <v>92</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C61" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C62" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="80" x14ac:dyDescent="0.2">
-      <c r="A62" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B62" s="6" t="s">
+    <row r="64" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B64" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C62" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C63" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C64" t="s">
-        <v>89</v>
+      <c r="C64" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="C65" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>27</v>
+        <v>87</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C67" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C68" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C69" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C70" t="s">
         <v>29</v>
@@ -2132,10 +2148,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C71" t="s">
         <v>29</v>
@@ -2143,10 +2159,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C72" t="s">
         <v>29</v>
@@ -2154,10 +2170,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C73" t="s">
         <v>29</v>
@@ -2165,59 +2181,81 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
-        <v>68</v>
+        <v>76</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="C74" t="s">
-        <v>124</v>
+        <v>29</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
-        <v>98</v>
+        <v>76</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="C75" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="64" x14ac:dyDescent="0.2">
-      <c r="A79" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B79" s="9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+      <c r="C76" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C77" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="64" x14ac:dyDescent="0.2">
       <c r="A81" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A82" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="B81" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" s="6" t="s">
-        <v>130</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" s="6" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
initial c++ for 3DAR1
need to add pars & map and rho in c++
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grantadams/Documents/GitHub/Rceattle/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grant.adams\GitHub\Rceattle ecosystem\Rceattle\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0A6E23-7146-7249-BECD-2D0D2B1F9B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C59BD4-347B-4D38-A803-5ADBAC992B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data_names" sheetId="1" r:id="rId1"/>
@@ -86,9 +86,6 @@
   </si>
   <si>
     <t>Description</t>
-  </si>
-  <si>
-    <t>Total catch in weight (kg) or numbers data</t>
   </si>
   <si>
     <t>Aging error matrices. Can have only one per species.</t>
@@ -557,6 +554,9 @@
     <t>Composition data distribution:
 0 = full multinomial
 1 = dirichlet-multinomial</t>
+  </si>
+  <si>
+    <t>Total catch in weight (mt) or numbers data</t>
   </si>
 </sst>
 </file>
@@ -1396,21 +1396,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F87"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.83203125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="119.5" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="119.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
@@ -1419,843 +1419,843 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" s="6" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="6" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
-        <v>75</v>
-      </c>
       <c r="B17" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C18" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="165" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C26" t="s">
+        <v>135</v>
+      </c>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" t="s">
+        <v>149</v>
+      </c>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" t="s">
+        <v>150</v>
+      </c>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C39" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A22" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" s="6" t="s">
+      <c r="C43" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C44" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C48" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="176" x14ac:dyDescent="0.2">
-      <c r="A25" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C26" t="s">
-        <v>136</v>
-      </c>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="C27" t="s">
-        <v>150</v>
-      </c>
-      <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="C28" t="s">
-        <v>151</v>
-      </c>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" t="s">
-        <v>145</v>
-      </c>
-      <c r="E31" s="2"/>
-    </row>
-    <row r="32" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="E32" s="2"/>
-    </row>
-    <row r="33" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A33" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="64" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B34" s="6" t="s">
+      <c r="C49" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="E35" s="2"/>
-    </row>
-    <row r="36" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A36" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="C52" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" t="s">
         <v>158</v>
       </c>
-      <c r="E36" s="2"/>
-    </row>
-    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E37" s="2"/>
-    </row>
-    <row r="38" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A38" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C40" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C41" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="112" x14ac:dyDescent="0.2">
-      <c r="A42" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E45" s="2"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C46" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A47" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C48" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="48" x14ac:dyDescent="0.2">
-      <c r="A49" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B50" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C50" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C51" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C52" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C53" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C54" t="s">
         <v>69</v>
       </c>
-      <c r="C54" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C55" t="s">
         <v>142</v>
       </c>
-      <c r="C55" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C56" t="s">
         <v>67</v>
       </c>
-      <c r="C56" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C58" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C60" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="48" x14ac:dyDescent="0.2">
-      <c r="A59" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="6" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C61" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C61" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C65" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C67" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C68" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C69" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C70" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C71" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C72" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C73" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C74" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C75" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C76" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C77" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="210" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B81" s="9" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C77" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" ht="192" x14ac:dyDescent="0.2">
-      <c r="A78" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" ht="64" x14ac:dyDescent="0.2">
-      <c r="A81" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B81" s="9" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="6" t="s">
         <v>127</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" s="6" t="s">
-        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Document schema gaps and remove the dead accumulation-age feature
Flip the 16 used-but-undocumented fleet_control/bioenergetics columns to
meta = TRUE so they appear in the generated meta_data_names.xlsx, and
regenerate the workbook from the schema.

Accumulation_age_lower/upper were only range-validated in data_check() and
never applied to composition data (no grouping exists in R or the C++
template), so the feature was dead and its docs were misleading. Remove the
validation, drop both spellings (incl. the Acuumulation typo) from the
roxygen field dictionary, and soft-deprecate the columns in switch_check():
an old workbook carrying either name is dropped once with a message.

Golden bit-identical across BS2017 SS/MS and GOA2018 SS/MS.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -798,12 +798,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>N_sel_bins</t>
+          <t>Selectivity_dimension</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Number of age or length bins to estimate non-parametric selectivity for Selectivity = 2 &amp; 5. Not used otherwise</t>
+          <t>"Age" or "Length".</t>
         </is>
       </c>
     </row>
@@ -815,12 +815,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sel_curve_pen1</t>
+          <t>N_sel_bins</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 1st penalty on selectivity.</t>
+          <t>Number of age or length bins to estimate non-parametric selectivity for Selectivity = 2 &amp; 5. Not used otherwise</t>
         </is>
       </c>
     </row>
@@ -832,12 +832,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sel_curve_pen2</t>
+          <t>Sel_curve_pen1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
+          <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 1st penalty on selectivity.</t>
         </is>
       </c>
     </row>
@@ -849,10 +849,44 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>Sel_curve_pen2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>If selectivity is set to type = 2 or 7 (non-parametric) this value will be the 2nd penalty on selectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sel_curve_pen3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Deviation-magnitude penalty weight (Sel_curve_pen3) for non-parametric / LogisticPM selectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>Time_varying_sel</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Wether a time-varying selectivity should be estimated for logistic, double logistic selectivity,  descending logistic , or non-parametric (Selectivity = 5). _x000D_
 0 = no_x000D_
@@ -863,40 +897,6 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Time_varying_sel_sd</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>The fixed or initial sd to use for time varying selectivity if set to 1, 4, or 5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Bin_first_selected</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Age/length bin at which selectivity becomes non-zero</t>
-        </is>
-      </c>
-    </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -905,10 +905,214 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>Time_varying_sel_sd</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The fixed or initial sd to use for time varying selectivity if set to 1, 4, or 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Sel_start_year</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>First year the fleet's time-varying selectivity deviations are estimated and penalized (NA -&gt; earliest year of data across fleets sharing the Selectivity_index, bounded below by styr).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Bin_first_selected</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Age/length bin at which selectivity becomes non-zero</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Sel_shape_sd</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Shape/smoothness selectivity penalty expressed as a standard deviation (an intuitive alternative to Sel_curve_pen1); weight = 1/(2*sd^2). NonParametric (2/9) and LogisticPM (11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sel_curvature_sd</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2nd-difference curvature selectivity penalty expressed as a standard deviation (Sel_curve_pen2); NonParametric-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sel_devmag_sd</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Deviation-magnitude selectivity penalty expressed as a standard deviation (Sel_curve_pen3). NonParametric (2/9) and LogisticPM (11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sel_shape_dir</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Direction of the (directional-mode) NonParametric shape penalty when Sel_shape_sd is used: "Decreasing" (default) or "Increasing".</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sel_pen_first_bin</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>First bin (age or length) for the non-parametric shape penalty (NA -&gt; Bin_first_selected).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sel_pen_last_bin</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Last (left) bin of the shape-penalty pairs (NA -&gt; nbins-2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Sel_shape_mode</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Shape-penalty mode: "Directional" (default) or "Smooth" (two-sided d^2, RTMB).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sel_avgsel_pen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Weight on the AMAK avgsel base-level penalty (type 9); 0 = off (default), 10 matches AMAK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sel_cap_bin</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NonParametricRPM bin cap (NA -&gt; no cap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>Sel_norm_bin1</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Age/length bin at which selectivity = 1. _x000D_
 If NA, it will not normalize selectivity. _x000D_
@@ -916,35 +1120,35 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>Sel_norm_bin2</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Upper age/length bin for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Age_max_selected` and `Age_max_selected_upper`</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
         <is>
           <t>Comp_loglike</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Composition data distribution:_x000D_
 -1 = AFSC multinomial_x000D_
@@ -953,36 +1157,36 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>Comp_weights</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Composition weights for composition likelihood. _x000D_
 After running model, these will update to McAllister &amp; Ianelli 1997 weights using the harmonic mean.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
         <is>
           <t>CAAL_loglike</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Composition data distribution:_x000D_
 0 = full multinomial_x000D_
@@ -990,104 +1194,104 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>CAAL_weights</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Composition weights for CAAL  likelihood.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>weight1_Numbers2</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>1 = catch/index is weight (kg) the observation _x000D_
 2 = catch/index is in numbers</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Weight_index</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Weight index to use for calculation of derived quantities</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>Age_transition_index</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>Age transition matrix (e.g. growth trajectory) index to used convert age to length</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>Q_index</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>index to use if catchability coefficients are to be set the same</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>Catchability</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>0 = fixed at "Q_sd_prior" _x000D_
 1 = Estimate as free parameter; _x000D_
@@ -1099,52 +1303,52 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>Q_init</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Starting value or fixed value for catchability</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
         <is>
           <t>Q_sd_prior</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Standard deviation for q prior</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>Time_varying_q</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>0 = no_x000D_
 1 = penalized deviate or random effect _x000D_
@@ -1155,35 +1359,35 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>Time_varying_q_sd</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>starting or fixed sd to use for the random walk of time varying q if set to 1</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>Estimate_index_sd</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>0 = use input "Log_sd" from index_data_x000D_
 1 = estimate as free parameter_x000D_
@@ -1191,35 +1395,35 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t>Index_sd</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Starting value to be used if "Estimate_index_sd" = 1</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>Estimate_catch_sd</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>0 = use input "Log_sd" from catch_data_x000D_
 1 = estimate as free parameter_x000D_
@@ -1227,186 +1431,220 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
         <is>
           <t>Catch_sd</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Starting value to be used if Estimate_catch_sd = 1</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Index_loglike</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Survey/index biomass observation likelihood family. 0 or "Lognormal" (default) = independent lognormal; "MVN"/"MVNORM" use a multivariate normal with a user-supplied covariance in index_cov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Observation month for the fleet (0 = not specified).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
         <is>
           <t>proj_F_prop</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>The proportion of future fishing mortality assigned to this fleet</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>index_data</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>Survey index or fishery indices in weight (kg) or numbers.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>catch_data</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>Total catch in weight (mt) or numbers data</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>comp_data</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>Survey/fishery age or length composition data. Note if sex is 3, put female composition data then male composition data (similar to SS).</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>caal_data</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>Survey/fishery CAAL data. Note if sex is 3, put female CAAL data then male CAAL data (similar to SS).</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>emp_sel</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Empirical/fixed selectivity for surveys and fisheries (leave empty if not used)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t>age_trans_matrix</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>Age transition matrix (e.g. growth trajectory) used to convert age to length for length comp data. _x000D_
 Can have multiple matrices for a species specified by Age_transition_index.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>age_error</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>Aging error matrices. Can have only one per species.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+    <row r="73">
+      <c r="A73" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Time-invariant or -varying empirical weight-at-age for calculation of derived quantities (SSB, Consumption/Ration, Suitability, Total Catch, Survey Biomass, etc). _x000D_
 Can have multiple weight-at-age data-sets for each species.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>maturity</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>Maturity-at-age for each species</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>sex_ratio</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Percent female at age for each species</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>M1_base</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>Residual natural mortality for each species</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>Ceq</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: _x000D_
 1 = Exponential (Stewart et al 1983)_x000D_
@@ -1416,224 +1654,258 @@
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>Cindex</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>Integer: which environmental index in env_data to use to drive bioenergetics</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Pvalue</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>Numeric: this scales the maximum consumption used for ration for each species; Pvalue is in Cmax*fT*Pvalue*Pyrs</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="80">
+      <c r="A80" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>fday</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>Numeric: number of foraging days per year for each species</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>Intercept of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>CB</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>Slope of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>Qc</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>Tco</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>Tcm</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>Tcl</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>CK1</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>CK4</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>bioenergetics_control</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Diet_loglike</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Diet composition likelihood distribution per predator species (0 = multinomial).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>bioenergetics_control</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Diet_comp_weights</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Diet composition weight (multinomial multiplier) per predator species.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>env_data</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Environmental indices such as bottom temperature data to incorporate into ration equation specificed by Ceq and Cindex. Also used to drive catchability if Estimate_q = 5 or 6. Will use the mean for missing years. Temperature should be in celcius.</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
+    <row r="92">
+      <c r="A92" t="inlineStr">
         <is>
           <t>ration_data</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>Annual relative foraging rate by age. Multiplied by pvalue and fday to scale maximum consumption to the number of days in a year that foraging occurs.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+    <row r="93">
+      <c r="A93" t="inlineStr">
         <is>
           <t>diet_data</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Multiple diet-data formats can be included:_x000D_
 _x000D_
@@ -1648,36 +1920,36 @@
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>NOTE: Most objects are ordered by species code if not specified</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
+    <row r="95">
+      <c r="A95" t="inlineStr">
         <is>
           <t>NOTE: Lengths are index 1 through nlenths</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
+    <row r="97">
+      <c r="A97" t="inlineStr">
         <is>
           <t>NOTE: For catch, index, and comp data, if "Year" is negative, it will predict for that year, but not include the data in the likelihood.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
+    <row r="98">
+      <c r="A98" t="inlineStr">
         <is>
           <t>NOTE: For emp_sel, weight, and ration_data, if "Year" == 0, those data will be used for all years</t>
         </is>

</xml_diff>

<commit_message>
Rename the catchability fleet_control columns to Catchability_*
Q_index -> Catchability_index, Q_init -> Catchability_init, and
Q_sd_prior -> Catchability_prior_sd, migrating the whole q family to the
descriptive Catchability_* naming. Each old name is kept as a schema alias and
upgraded in place by .rce_upgrade_fleet_control_aliases(), so existing data
lists, .rda, and workbooks keep fitting identically. Update every consumer
(build_params, build_map, rearrange_data, data_check, combine_data, the data
class printer), add the alias upgrade to data_check/combine_data/rearrange_data
so standalone calls on legacy data also work, refresh globalVariables(), the
alias-pin test, the roxygen field labels, and the generated meta workbook.
Bundled .rda keep the old names for now (regenerated onto canonical names in a
later step); the runtime upgrade makes fits bit-identical meanwhile.

Golden bit-identical across BS2017 SS/MS and GOA2018 SS/MS.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Q_index</t>
+          <t>Catchability_index</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Q_init</t>
+          <t>Catchability_init</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Q_sd_prior</t>
+          <t>Catchability_prior_sd</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">

</xml_diff>

<commit_message>
Rename Sel_norm_bin1/2, weight1_Numbers2, and proj_F_prop columns
Four more intuitive fleet_control column names, each keeping a back-compat
schema alias upgraded in place by .rce_upgrade_fleet_control_aliases():
 - Sel_norm_bin1     -> Sel_norm_bin
 - Sel_norm_bin2     -> Sel_norm_bin_upper
 - weight1_Numbers2  -> Observation_units  (drives both catch and index
   prediction; the alias accepts BOTH the documented lowercase spelling and
   the capital Weight1_Numbers2 the data/consumers actually used, closing a
   latent case mismatch)
 - proj_F_prop       -> Proj_F_proportion  (the fleet_control COLUMN only; the
   identically named TMB parameter/map/phase/dictionary keep proj_F_prop, so
   the C++ template is untouched)

Update every consumer, regenerate the three bundled datasets to canonical
(values byte-identical), the meta workbook, the alias-pin test, and roxygen.

Golden bit-identical across BS2017 SS/MS and GOA2018 SS/MS.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Sel_norm_bin1</t>
+          <t>Sel_norm_bin</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1128,12 +1128,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Sel_norm_bin2</t>
+          <t>Sel_norm_bin_upper</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Upper age/length bin for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Age_max_selected` and `Age_max_selected_upper`</t>
+          <t>Upper age/length bin for selectivity normalization (default = NA). If NA, does not use the age range, If not NA, uses mean selectivity between `Sel_norm_bin` and `Sel_norm_bin_upper`</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>weight1_Numbers2</t>
+          <t>Observation_units</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>proj_F_prop</t>
+          <t>Proj_F_proportion</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">

</xml_diff>

<commit_message>
Add composition tail accumulation (AFSC ac_yng / ac_old)
New Comp_accum_young / Comp_accum_old fleet_control columns fold the
young/old composition tails into a boundary bin before the likelihood,
per sex block for joint-sex comps, for every composition family
(including the default MultinomialAFSC). No-op by default -> existing
models bit-identical.

Registered in the canonical schema (switch_check materialization,
data.R docs, meta workbook); data_check() rejects out-of-range or
inverted (young > old) bins; build_osa_data() refuses an active
accumulation (OSA residuals use the un-accumulated bins -- a consistent
OSA path is a planned follow-up). Folding is verified against a
from-scratch AFSC NLL for combined- and joint-sex comps; golden
reference bit-identical across the four BS/GOA models.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1219,50 +1219,50 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>Comp_accum_young</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Age/length composition young-tail accumulation bin (AFSC ac_yng): a 1-based ordinal on the fleet's composition dimension; bins below it are folded into it before the likelihood. NA or 1 = no young accumulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Comp_accum_old</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Age/length composition old-tail accumulation bin (AFSC ac_old): a 1-based ordinal on the fleet's composition dimension; bins above it are folded into it before the likelihood. NA, 0, or a value &gt;= the number of bins = no old accumulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>Observation_units</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>1 = catch/index is weight (kg) the observation _x000D_
 2 = catch/index is in numbers</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Weight_index</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Weight index to use for calculation of derived quantities</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Age_transition_index</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Age transition matrix (e.g. growth trajectory) index to used convert age to length</t>
-        </is>
-      </c>
-    </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Catchability_index</t>
+          <t>Weight_index</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>index to use if catchability coefficients are to be set the same</t>
+          <t>Weight index to use for calculation of derived quantities</t>
         </is>
       </c>
     </row>
@@ -1288,10 +1288,44 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
+          <t>Age_transition_index</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Age transition matrix (e.g. growth trajectory) index to used convert age to length</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Catchability_index</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>index to use if catchability coefficients are to be set the same</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>Catchability</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Catchability form. Accepts integer codes or readable strings:_x000D_
 0 or "Fixed" = fixed at Catchability_init_x000D_
@@ -1305,40 +1339,6 @@
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Catchability_init</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Starting value or fixed value for catchability</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Catchability_prior_sd</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Standard deviation for q prior</t>
-        </is>
-      </c>
-    </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
@@ -1347,10 +1347,44 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>Catchability_init</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Starting value or fixed value for catchability</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Catchability_prior_sd</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Standard deviation for q prior</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>Time_varying_q</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>0 = no_x000D_
 1 = penalized deviate or random effect _x000D_
@@ -1361,35 +1395,35 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t>Time_varying_q_sd</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>starting or fixed sd to use for the random walk of time varying q if set to 1</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>Estimate_index_sd</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>0 = use input "Log_sd" from index_data_x000D_
 1 = estimate as free parameter_x000D_
@@ -1397,35 +1431,35 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
         <is>
           <t>Index_sd</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Starting value to be used if "Estimate_index_sd" = 1</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>Estimate_catch_sd</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>0 = use input "Log_sd" from catch_data_x000D_
 1 = estimate as free parameter_x000D_
@@ -1433,40 +1467,6 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Catch_sd</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Starting value to be used if Estimate_catch_sd = 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>fleet_control</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Index_distribution</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Survey/index biomass observation likelihood family. 0 or "Lognormal" (default) = independent lognormal; "MVN"/"MVNORM" use a multivariate normal with a user-supplied covariance in index_cov.</t>
-        </is>
-      </c>
-    </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
@@ -1475,12 +1475,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>Catch_sd</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Observation month for the fleet (0 = not specified).</t>
+          <t>Starting value to be used if Estimate_catch_sd = 1</t>
         </is>
       </c>
     </row>
@@ -1492,161 +1492,195 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Proj_F_proportion</t>
+          <t>Index_distribution</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The proportion of future fishing mortality assigned to this fleet</t>
+          <t>Survey/index biomass observation likelihood family. 0 or "Lognormal" (default) = independent lognormal; "MVN"/"MVNORM" use a multivariate normal with a user-supplied covariance in index_cov.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>index_data</t>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Month</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Survey index or fishery indices in weight (kg) or numbers.</t>
+          <t>Observation month for the fleet (0 = not specified).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>catch_data</t>
+          <t>fleet_control</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Proj_F_proportion</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Total catch in weight (mt) or numbers data</t>
+          <t>The proportion of future fishing mortality assigned to this fleet</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>comp_data</t>
+          <t>index_data</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Survey/fishery age or length composition data. Note if sex is 3, put female composition data then male composition data (similar to SS).</t>
+          <t>Survey index or fishery indices in weight (kg) or numbers.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>caal_data</t>
+          <t>catch_data</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Survey/fishery CAAL data. Note if sex is 3, put female CAAL data then male CAAL data (similar to SS).</t>
+          <t>Total catch in weight (mt) or numbers data</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>emp_sel</t>
+          <t>comp_data</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Empirical/fixed selectivity for surveys and fisheries (leave empty if not used)</t>
+          <t>Survey/fishery age or length composition data. Note if sex is 3, put female composition data then male composition data (similar to SS).</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>caal_data</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Survey/fishery CAAL data. Note if sex is 3, put female CAAL data then male CAAL data (similar to SS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>emp_sel</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Empirical/fixed selectivity for surveys and fisheries (leave empty if not used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>age_trans_matrix</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Age transition matrix (e.g. growth trajectory) used to convert age to length for length comp data. _x000D_
 Can have multiple matrices for a species specified by Age_transition_index.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>age_error</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>Aging error matrices. Can have only one per species.</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Time-invariant or -varying empirical weight-at-age for calculation of derived quantities (SSB, Consumption/Ration, Suitability, Total Catch, Survey Biomass, etc). _x000D_
 Can have multiple weight-at-age data-sets for each species.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>maturity</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Maturity-at-age for each species</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>sex_ratio</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Percent female at age for each species</t>
-        </is>
-      </c>
-    </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>M1_base</t>
+          <t>maturity</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Residual natural mortality for each species</t>
+          <t>Maturity-at-age for each species</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>sex_ratio</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Percent female at age for each species</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>M1_base</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Residual natural mortality for each species</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t>bioenergetics_control</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Ceq</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>Integer: switch for which bioenergetics equation to use for each species for ft to scale max consumtion: _x000D_
 1 = Exponential (Stewart et al 1983)_x000D_
@@ -1656,40 +1690,6 @@
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>bioenergetics_control</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Cindex</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Integer: which environmental index in env_data to use to drive bioenergetics</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>bioenergetics_control</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Pvalue</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Numeric: this scales the maximum consumption used for ration for each species; Pvalue is in Cmax*fT*Pvalue*Pyrs</t>
-        </is>
-      </c>
-    </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
@@ -1698,12 +1698,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>fday</t>
+          <t>Cindex</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Numeric: number of foraging days per year for each species</t>
+          <t>Integer: which environmental index in env_data to use to drive bioenergetics</t>
         </is>
       </c>
     </row>
@@ -1715,12 +1715,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>Pvalue</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Intercept of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
+          <t>Numeric: this scales the maximum consumption used for ration for each species; Pvalue is in Cmax*fT*Pvalue*Pyrs</t>
         </is>
       </c>
     </row>
@@ -1732,12 +1732,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>fday</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Slope of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
+          <t>Numeric: number of foraging days per year for each species</t>
         </is>
       </c>
     </row>
@@ -1749,12 +1749,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Qc</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
+          <t>Intercept of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1766,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tco</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
+          <t>Slope of allometric mass function for calculating maximum consumption: CA * Weight ^ CB</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Tcm</t>
+          <t>Qc</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Tcl</t>
+          <t>Tco</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>CK1</t>
+          <t>Tcm</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>CK4</t>
+          <t>Tcl</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1851,12 +1851,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Diet_distribution</t>
+          <t>CK1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Diet composition likelihood distribution per predator species (0 = multinomial).</t>
+          <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
@@ -1868,46 +1868,80 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Diet_comp_weights</t>
+          <t>CK4</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Diet composition weight (multinomial multiplier) per predator species.</t>
+          <t>Parameter for temperature scaling function of maximum consumption specified by Ceq</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>env_data</t>
+          <t>bioenergetics_control</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Diet_distribution</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Environmental indices such as bottom temperature data to incorporate into ration equation specificed by Ceq and Cindex. Also used to drive catchability if Catchability = 5 or 6. Will use the mean for missing years. Temperature should be in celcius.</t>
+          <t>Diet composition likelihood distribution per predator species (0 = multinomial).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ration_data</t>
+          <t>bioenergetics_control</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Diet_comp_weights</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Annual relative foraging rate by age. Multiplied by pvalue and fday to scale maximum consumption to the number of days in a year that foraging occurs.</t>
+          <t>Diet composition weight (multinomial multiplier) per predator species.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>env_data</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Environmental indices such as bottom temperature data to incorporate into ration equation specificed by Ceq and Cindex. Also used to drive catchability if Catchability = 5 or 6. Will use the mean for missing years. Temperature should be in celcius.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ration_data</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Annual relative foraging rate by age. Multiplied by pvalue and fday to scale maximum consumption to the number of days in a year that foraging occurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>diet_data</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Stomach proportion by weight for each predator, prey, predator age, prey age combination. Multiple diet-data formats can be included:_x000D_
 _x000D_
@@ -1922,36 +1956,36 @@
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>NOTE: Most objects are ordered by species code if not specified</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>NOTE: Lengths are index 1 through nlenths</t>
-        </is>
-      </c>
-    </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
+          <t>NOTE: Most objects are ordered by species code if not specified</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>NOTE: For catch, index, and comp data, if "Year" is negative, it will predict for that year, but not include the data in the likelihood.</t>
+          <t>NOTE: Lengths are index 1 through nlenths</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
+        <is>
+          <t>NOTE: Columns for ages are index by 1 trhough nages, but are place holders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>NOTE: For catch, index, and comp data, if "Year" is negative, it will predict for that year, but not include the data in the likelihood.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>NOTE: For emp_sel, weight, and ration_data, if "Year" == 0, those data will be used for all years</t>
         </is>

</xml_diff>

<commit_message>
Accept string aliases for Diet_distribution (5.1.1)
Diet_distribution was the one composition-likelihood switch that took only the integer
code, unlike Comp_distribution / CAAL_distribution which accept string aliases via
comp_loglike_map. Add a diet-specific map (Multinomial = 0, DirichletMultinomial = 1 --
the diet likelihood has no AFSC variant, so no -1), wire it into switch_check via
.map_switch, and set allowed = "diet_loglike_map" on the schema column. Integer input
still passes through unchanged; an unsupported value (e.g. "MultinomialAFSC") errors
with the valid options.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1891,7 +1891,9 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Diet composition likelihood distribution per predator species (0 = multinomial).</t>
+          <t>Diet composition likelihood distribution per predator species:_x000D_
+0 = multinomial_x000D_
+1 = dirichlet-multinomial</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten the reweighting and linkage prose
Editing pass on the user-facing text from the last two commits.

reweight_comps(): the help page led with three paragraphs of description where
one belongs, and put the parameter-versus-column mechanism ahead of what the
function does. Description is now a single paragraph; the mechanism, the
skipped fleets and the convergence rule move to details.

NEWS: cut the asides, split the six-process entry so the three refusals are
their own paragraph, and describe the intercept init in terms a reader can act
on -- a catchability of 0.8, a von Bertalanffy K of 0.25 -- rather than a list
of internal parameter names.

Comp_weights dictionary entry: says what the weight does under each likelihood
in two short lines, and points at Comp_weights_mcallister and reweight_comps()
rather than explaining warm starts. Meta workbook regenerated to match.
</commit_message>
<xml_diff>
--- a/inst/extdata/meta_data_names.xlsx
+++ b/inst/extdata/meta_data_names.xlsx
@@ -1171,8 +1171,9 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Starting composition weight, used when a model is built from scratch; a fit warm-started from `inits` carries the parameter forward instead. _x000D_
-A fitted model reports the implied McAllister &amp; Ianelli (1997) harmonic-mean weight separately, in `Comp_weights_mcallister`; `reweight_comps()` iterates on it.</t>
+          <t>Composition weight. Multiplies the input sample size under a multinomial likelihood; starts the estimated weight under a Dirichlet-multinomial. _x000D_
+Read when a model is built from scratch -- a refit keeps the weight it is given. _x000D_
+See 'Comp_weights_mcallister' for the weight a fit implies, and reweight_comps() to tune towards it.</t>
         </is>
       </c>
     </row>

</xml_diff>